<commit_message>
test: make Excel reader tests independent of input row order
</commit_message>
<xml_diff>
--- a/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
+++ b/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ENM\Programming\Repositories\software_BioPot-Gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A687F830-EA5B-4EFB-905A-3B3E100C19F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9263D1-AB46-4953-B486-CF275CE4C562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24" yWindow="-12528" windowWidth="22296" windowHeight="11904" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_INFORMATIVO" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="323">
   <si>
     <t>BioPot-Gas v0.6 | Informativo do template</t>
   </si>
@@ -999,6 +999,18 @@
   </si>
   <si>
     <t>Alerta para eficiência experimental acima de 100%</t>
+  </si>
+  <si>
+    <t>WATER</t>
+  </si>
+  <si>
+    <t>water</t>
+  </si>
+  <si>
+    <t>H2O</t>
+  </si>
+  <si>
+    <t>Available water, treated separately from organic substrates</t>
   </si>
 </sst>
 </file>
@@ -1032,7 +1044,7 @@
       <name val="Carlito"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1089,6 +1101,18 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -1109,7 +1133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1144,9 +1168,6 @@
     <xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1165,19 +1186,31 @@
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1428,7 +1461,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N26"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" style="9" customWidth="1"/>
@@ -1620,15 +1653,28 @@
         <v>26</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="114">
-      <c r="A18" s="14" t="s">
+    <row r="18" spans="1:14">
+      <c r="A18" s="29" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="60">
-      <c r="A19" s="3" t="s">
+    <row r="19" spans="1:14" ht="15">
+      <c r="A19" s="28" t="s">
         <v>53</v>
       </c>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
+      <c r="E19" s="28"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
+      <c r="H19" s="28"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="28"/>
+      <c r="K19" s="28"/>
+      <c r="L19" s="28"/>
+      <c r="M19" s="28"/>
+      <c r="N19" s="28"/>
     </row>
     <row r="20" spans="1:14" ht="15">
       <c r="A20" s="5" t="s">
@@ -1674,41 +1720,43 @@
         <v>67</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
-      <c r="A21" s="8" t="s">
-        <v>68</v>
-      </c>
-      <c r="B21" s="8" t="s">
-        <v>69</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D21" s="8">
+    <row r="21" spans="1:14" s="25" customFormat="1" ht="28.5">
+      <c r="A21" s="26" t="s">
+        <v>319</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>320</v>
+      </c>
+      <c r="C21" s="27" t="b">
+        <v>0</v>
+      </c>
+      <c r="D21" s="26">
+        <v>0</v>
+      </c>
+      <c r="E21" s="26" t="s">
+        <v>321</v>
+      </c>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
+      <c r="I21" s="26"/>
+      <c r="J21" s="26"/>
+      <c r="K21" s="26" t="s">
+        <v>319</v>
+      </c>
+      <c r="L21" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="M21" s="26" t="s">
+        <v>322</v>
+      </c>
+      <c r="N21" s="27" t="b">
         <v>1</v>
-      </c>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="L21" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="M21" s="8" t="s">
-        <v>72</v>
-      </c>
-      <c r="N21" s="8" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="8" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B22" s="8" t="s">
         <v>69</v>
@@ -1717,7 +1765,7 @@
         <v>36</v>
       </c>
       <c r="D22" s="8">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
@@ -1740,16 +1788,16 @@
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="C23" s="8" t="s">
         <v>36</v>
       </c>
       <c r="D23" s="8">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E23" s="8"/>
       <c r="F23" s="8"/>
@@ -1770,18 +1818,18 @@
         <v>36</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="28.5">
+    <row r="24" spans="1:14">
       <c r="A24" s="8" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D24" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E24" s="8"/>
       <c r="F24" s="8"/>
@@ -1796,49 +1844,47 @@
         <v>71</v>
       </c>
       <c r="M24" s="8" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="N24" s="8" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" ht="28.5">
       <c r="A25" s="8" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D25" s="8">
-        <v>0</v>
-      </c>
-      <c r="E25" s="8" t="s">
-        <v>81</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="E25" s="8"/>
       <c r="F25" s="8"/>
       <c r="G25" s="8"/>
       <c r="H25" s="8"/>
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="L25" s="8" t="s">
-        <v>83</v>
+        <v>71</v>
       </c>
       <c r="M25" s="8" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="N25" s="8" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="26" spans="1:14">
       <c r="A26" s="8" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>80</v>
@@ -1849,24 +1895,16 @@
       <c r="D26" s="8">
         <v>0</v>
       </c>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8">
-        <v>6</v>
-      </c>
-      <c r="G26" s="8">
-        <v>10</v>
-      </c>
-      <c r="H26" s="8">
-        <v>5</v>
-      </c>
-      <c r="I26" s="8">
-        <v>0</v>
-      </c>
-      <c r="J26" s="8">
-        <v>0</v>
-      </c>
+      <c r="E26" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
       <c r="K26" s="8" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="L26" s="8" t="s">
         <v>83</v>
@@ -1878,12 +1916,281 @@
         <v>39</v>
       </c>
     </row>
+    <row r="27" spans="1:14">
+      <c r="A27" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D27" s="8">
+        <v>0</v>
+      </c>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8">
+        <v>6</v>
+      </c>
+      <c r="G27" s="8">
+        <v>10</v>
+      </c>
+      <c r="H27" s="8">
+        <v>5</v>
+      </c>
+      <c r="I27" s="8">
+        <v>0</v>
+      </c>
+      <c r="J27" s="8">
+        <v>0</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>86</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="M27" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="N27" s="8" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14">
+      <c r="A28" s="30"/>
+      <c r="B28" s="30"/>
+      <c r="C28" s="30"/>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30"/>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
+      <c r="K28" s="30"/>
+      <c r="L28" s="30"/>
+      <c r="M28" s="30"/>
+      <c r="N28" s="30"/>
+    </row>
+    <row r="29" spans="1:14">
+      <c r="A29" s="30"/>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
+      <c r="D29" s="30"/>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+      <c r="K29" s="30"/>
+      <c r="L29" s="30"/>
+      <c r="M29" s="30"/>
+      <c r="N29" s="30"/>
+    </row>
+    <row r="30" spans="1:14">
+      <c r="A30" s="30"/>
+      <c r="B30" s="30"/>
+      <c r="C30" s="30"/>
+      <c r="D30" s="30"/>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30"/>
+      <c r="I30" s="30"/>
+      <c r="J30" s="30"/>
+      <c r="K30" s="30"/>
+      <c r="L30" s="30"/>
+      <c r="M30" s="30"/>
+      <c r="N30" s="30"/>
+    </row>
+    <row r="31" spans="1:14">
+      <c r="A31" s="30"/>
+      <c r="B31" s="30"/>
+      <c r="C31" s="30"/>
+      <c r="D31" s="30"/>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30"/>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30"/>
+      <c r="K31" s="30"/>
+      <c r="L31" s="30"/>
+      <c r="M31" s="30"/>
+      <c r="N31" s="30"/>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" s="30"/>
+      <c r="B32" s="30"/>
+      <c r="C32" s="30"/>
+      <c r="D32" s="30"/>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
+      <c r="J32" s="30"/>
+      <c r="K32" s="30"/>
+      <c r="L32" s="30"/>
+      <c r="M32" s="30"/>
+      <c r="N32" s="30"/>
+    </row>
+    <row r="33" spans="1:14">
+      <c r="A33" s="30"/>
+      <c r="B33" s="30"/>
+      <c r="C33" s="30"/>
+      <c r="D33" s="30"/>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30"/>
+      <c r="I33" s="30"/>
+      <c r="J33" s="30"/>
+      <c r="K33" s="30"/>
+      <c r="L33" s="30"/>
+      <c r="M33" s="30"/>
+      <c r="N33" s="30"/>
+    </row>
+    <row r="34" spans="1:14">
+      <c r="A34" s="30"/>
+      <c r="B34" s="30"/>
+      <c r="C34" s="30"/>
+      <c r="D34" s="30"/>
+      <c r="E34" s="30"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30"/>
+      <c r="I34" s="30"/>
+      <c r="J34" s="30"/>
+      <c r="K34" s="30"/>
+      <c r="L34" s="30"/>
+      <c r="M34" s="30"/>
+      <c r="N34" s="30"/>
+    </row>
+    <row r="35" spans="1:14">
+      <c r="A35" s="30"/>
+      <c r="B35" s="30"/>
+      <c r="C35" s="30"/>
+      <c r="D35" s="30"/>
+      <c r="E35" s="30"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30"/>
+      <c r="I35" s="30"/>
+      <c r="J35" s="30"/>
+      <c r="K35" s="30"/>
+      <c r="L35" s="30"/>
+      <c r="M35" s="30"/>
+      <c r="N35" s="30"/>
+    </row>
+    <row r="36" spans="1:14">
+      <c r="A36" s="30"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="30"/>
+      <c r="D36" s="30"/>
+      <c r="E36" s="30"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30"/>
+      <c r="I36" s="30"/>
+      <c r="J36" s="30"/>
+      <c r="K36" s="30"/>
+      <c r="L36" s="30"/>
+      <c r="M36" s="30"/>
+      <c r="N36" s="30"/>
+    </row>
+    <row r="37" spans="1:14">
+      <c r="A37" s="30"/>
+      <c r="B37" s="30"/>
+      <c r="C37" s="30"/>
+      <c r="D37" s="30"/>
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30"/>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30"/>
+      <c r="K37" s="30"/>
+      <c r="L37" s="30"/>
+      <c r="M37" s="30"/>
+      <c r="N37" s="30"/>
+    </row>
+    <row r="38" spans="1:14">
+      <c r="A38" s="30"/>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
+      <c r="D38" s="30"/>
+      <c r="E38" s="30"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30"/>
+      <c r="I38" s="30"/>
+      <c r="J38" s="30"/>
+      <c r="K38" s="30"/>
+      <c r="L38" s="30"/>
+      <c r="M38" s="30"/>
+      <c r="N38" s="30"/>
+    </row>
+    <row r="39" spans="1:14">
+      <c r="A39" s="30"/>
+      <c r="B39" s="30"/>
+      <c r="C39" s="30"/>
+      <c r="D39" s="30"/>
+      <c r="E39" s="30"/>
+      <c r="F39" s="30"/>
+      <c r="G39" s="30"/>
+      <c r="H39" s="30"/>
+      <c r="I39" s="30"/>
+      <c r="J39" s="30"/>
+      <c r="K39" s="30"/>
+      <c r="L39" s="30"/>
+      <c r="M39" s="30"/>
+      <c r="N39" s="30"/>
+    </row>
+    <row r="40" spans="1:14">
+      <c r="A40" s="30"/>
+      <c r="B40" s="30"/>
+      <c r="C40" s="30"/>
+      <c r="D40" s="30"/>
+      <c r="E40" s="30"/>
+      <c r="F40" s="30"/>
+      <c r="G40" s="30"/>
+      <c r="H40" s="30"/>
+      <c r="I40" s="30"/>
+      <c r="J40" s="30"/>
+      <c r="K40" s="30"/>
+      <c r="L40" s="30"/>
+      <c r="M40" s="30"/>
+      <c r="N40" s="30"/>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" s="30"/>
+      <c r="B41" s="30"/>
+      <c r="C41" s="30"/>
+      <c r="D41" s="30"/>
+      <c r="E41" s="30"/>
+      <c r="F41" s="30"/>
+      <c r="G41" s="30"/>
+      <c r="H41" s="30"/>
+      <c r="I41" s="30"/>
+      <c r="J41" s="30"/>
+      <c r="K41" s="30"/>
+      <c r="L41" s="30"/>
+      <c r="M41" s="30"/>
+      <c r="N41" s="30"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:N19"/>
+  </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C21:C200 N21:N200" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" sqref="C22:C201 N22:N201" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="K21:K200" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="K22:K201" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"DATABASE,FORMULA,ELEMENTS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1903,108 +2210,108 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
     </row>
     <row r="2" spans="1:6" ht="15">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
     </row>
     <row r="3" spans="1:6" ht="15">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="15" t="s">
         <v>91</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
     </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="15" t="s">
+    <row r="4" spans="1:6" ht="28.5">
+      <c r="A4" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="15" t="str">
+      <c r="B4" s="14" t="str">
         <f>'01_INPUTS'!B4</f>
         <v>Example BioPot-Gas v0.5</v>
       </c>
-      <c r="C4" s="15"/>
+      <c r="C4" s="14"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B5" s="15" t="str">
+      <c r="B5" s="14" t="str">
         <f>'01_INPUTS'!B5</f>
         <v>Edgar Amaral Silveira</v>
       </c>
-      <c r="C5" s="15"/>
+      <c r="C5" s="14"/>
       <c r="D5" s="4"/>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="15" t="str">
+      <c r="B6" s="14" t="str">
         <f>'01_INPUTS'!B6</f>
         <v>2026-06-05</v>
       </c>
-      <c r="C6" s="15"/>
+      <c r="C6" s="14"/>
       <c r="D6" s="4"/>
       <c r="E6" s="4"/>
       <c r="F6" s="4"/>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="15" t="str">
+      <c r="B7" s="14" t="str">
         <f>'01_INPUTS'!B7</f>
         <v>kmol/h</v>
       </c>
-      <c r="C7" s="15"/>
+      <c r="C7" s="14"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="14"/>
+      <c r="C8" s="14"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
     </row>
     <row r="9" spans="1:6" ht="15">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
+      <c r="B9" s="20"/>
+      <c r="C9" s="20"/>
     </row>
     <row r="10" spans="1:6" ht="15">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="15" t="s">
         <v>89</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="15" t="s">
         <v>91</v>
       </c>
       <c r="D10" s="4"/>
@@ -2012,11 +2319,11 @@
       <c r="F10" s="4"/>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="15" t="s">
+      <c r="A11" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="15"/>
-      <c r="C11" s="15" t="s">
+      <c r="B11" s="14"/>
+      <c r="C11" s="14" t="s">
         <v>93</v>
       </c>
       <c r="D11" s="4"/>
@@ -2024,11 +2331,11 @@
       <c r="F11" s="4"/>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15" t="s">
+      <c r="B12" s="14"/>
+      <c r="C12" s="14" t="s">
         <v>94</v>
       </c>
       <c r="D12" s="4"/>
@@ -2036,11 +2343,11 @@
       <c r="F12" s="4"/>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15" t="s">
+      <c r="B13" s="14"/>
+      <c r="C13" s="14" t="s">
         <v>95</v>
       </c>
       <c r="D13" s="4"/>
@@ -2048,11 +2355,11 @@
       <c r="F13" s="4"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15" t="s">
+      <c r="B14" s="14"/>
+      <c r="C14" s="14" t="s">
         <v>96</v>
       </c>
       <c r="D14" s="4"/>
@@ -2060,11 +2367,11 @@
       <c r="F14" s="4"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15" t="s">
+      <c r="B15" s="14"/>
+      <c r="C15" s="14" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="4"/>
@@ -2091,11 +2398,11 @@
       <c r="F17" s="4"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="15" t="s">
+      <c r="A18" s="14" t="s">
         <v>101</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15" t="s">
+      <c r="B18" s="14"/>
+      <c r="C18" s="14" t="s">
         <v>102</v>
       </c>
       <c r="D18" s="4"/>
@@ -2103,31 +2410,31 @@
       <c r="F18" s="4"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="15"/>
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
       <c r="D19" s="4"/>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
     </row>
     <row r="20" spans="1:6" ht="15">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
       <c r="D20" s="4"/>
       <c r="E20" s="4"/>
       <c r="F20" s="4"/>
     </row>
     <row r="21" spans="1:6" ht="15">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B21" s="17" t="s">
+      <c r="B21" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="16" t="s">
         <v>91</v>
       </c>
       <c r="D21" s="4"/>
@@ -2135,11 +2442,11 @@
       <c r="F21" s="4"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="14" t="s">
         <v>104</v>
       </c>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15" t="s">
+      <c r="B22" s="14"/>
+      <c r="C22" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D22" s="4"/>
@@ -2147,11 +2454,11 @@
       <c r="F22" s="4"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="15" t="s">
+      <c r="A23" s="14" t="s">
         <v>106</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15" t="s">
+      <c r="B23" s="14"/>
+      <c r="C23" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D23" s="4"/>
@@ -2159,11 +2466,11 @@
       <c r="F23" s="4"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="15" t="s">
+      <c r="A24" s="14" t="s">
         <v>107</v>
       </c>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15" t="s">
+      <c r="B24" s="14"/>
+      <c r="C24" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D24" s="4"/>
@@ -2171,11 +2478,11 @@
       <c r="F24" s="4"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="14" t="s">
         <v>108</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15" t="s">
+      <c r="B25" s="14"/>
+      <c r="C25" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D25" s="4"/>
@@ -2202,11 +2509,11 @@
       <c r="F27" s="4"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="15" t="s">
+      <c r="A28" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="B28" s="15"/>
-      <c r="C28" s="15" t="s">
+      <c r="B28" s="14"/>
+      <c r="C28" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D28" s="4"/>
@@ -2214,31 +2521,31 @@
       <c r="F28" s="4"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="15"/>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="14"/>
+      <c r="C29" s="14"/>
       <c r="D29" s="4"/>
       <c r="E29" s="4"/>
       <c r="F29" s="4"/>
     </row>
     <row r="30" spans="1:6" ht="15">
-      <c r="A30" s="23" t="s">
+      <c r="A30" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
+      <c r="B30" s="22"/>
+      <c r="C30" s="22"/>
       <c r="D30" s="4"/>
       <c r="E30" s="4"/>
       <c r="F30" s="4"/>
     </row>
     <row r="31" spans="1:6" ht="15">
-      <c r="A31" s="17" t="s">
+      <c r="A31" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B31" s="17" t="s">
+      <c r="B31" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="16" t="s">
         <v>91</v>
       </c>
       <c r="D31" s="4"/>
@@ -2246,11 +2553,11 @@
       <c r="F31" s="4"/>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="15" t="s">
+      <c r="A32" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15" t="s">
+      <c r="B32" s="14"/>
+      <c r="C32" s="14" t="s">
         <v>114</v>
       </c>
       <c r="D32" s="4"/>
@@ -2258,11 +2565,11 @@
       <c r="F32" s="4"/>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="15" t="s">
+      <c r="A33" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15" t="s">
+      <c r="B33" s="14"/>
+      <c r="C33" s="14" t="s">
         <v>114</v>
       </c>
       <c r="D33" s="4"/>
@@ -2311,31 +2618,31 @@
       <c r="F37" s="4"/>
     </row>
     <row r="38" spans="1:6">
-      <c r="A38" s="15"/>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15"/>
+      <c r="A38" s="14"/>
+      <c r="B38" s="14"/>
+      <c r="C38" s="14"/>
       <c r="D38" s="4"/>
       <c r="E38" s="4"/>
       <c r="F38" s="4"/>
     </row>
     <row r="39" spans="1:6" s="9" customFormat="1" ht="15">
-      <c r="A39" s="23" t="s">
+      <c r="A39" s="22" t="s">
         <v>120</v>
       </c>
-      <c r="B39" s="23"/>
-      <c r="C39" s="23"/>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
       <c r="D39" s="4"/>
       <c r="E39" s="4"/>
       <c r="F39" s="4"/>
     </row>
     <row r="40" spans="1:6" ht="15">
-      <c r="A40" s="17" t="s">
+      <c r="A40" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B40" s="17" t="s">
+      <c r="B40" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="C40" s="16" t="s">
         <v>91</v>
       </c>
       <c r="D40" s="4"/>
@@ -2384,11 +2691,11 @@
       <c r="F44" s="4"/>
     </row>
     <row r="45" spans="1:6">
-      <c r="A45" s="15" t="s">
+      <c r="A45" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="B45" s="15"/>
-      <c r="C45" s="15" t="s">
+      <c r="B45" s="14"/>
+      <c r="C45" s="14" t="s">
         <v>122</v>
       </c>
       <c r="D45" s="4"/>
@@ -2396,11 +2703,11 @@
       <c r="F45" s="4"/>
     </row>
     <row r="46" spans="1:6">
-      <c r="A46" s="15" t="s">
+      <c r="A46" s="14" t="s">
         <v>127</v>
       </c>
-      <c r="B46" s="15"/>
-      <c r="C46" s="15" t="s">
+      <c r="B46" s="14"/>
+      <c r="C46" s="14" t="s">
         <v>128</v>
       </c>
       <c r="D46" s="4"/>
@@ -2408,31 +2715,31 @@
       <c r="F46" s="4"/>
     </row>
     <row r="47" spans="1:6">
-      <c r="A47" s="15"/>
-      <c r="B47" s="15"/>
-      <c r="C47" s="15"/>
+      <c r="A47" s="14"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
       <c r="D47" s="4"/>
       <c r="E47" s="4"/>
       <c r="F47" s="4"/>
     </row>
     <row r="48" spans="1:6" ht="15">
-      <c r="A48" s="23" t="s">
+      <c r="A48" s="22" t="s">
         <v>129</v>
       </c>
-      <c r="B48" s="23"/>
-      <c r="C48" s="23"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
       <c r="D48" s="4"/>
       <c r="E48" s="4"/>
       <c r="F48" s="4"/>
     </row>
     <row r="49" spans="1:6" ht="15">
-      <c r="A49" s="17" t="s">
+      <c r="A49" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B49" s="17" t="s">
+      <c r="B49" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C49" s="16" t="s">
         <v>91</v>
       </c>
       <c r="D49" s="4"/>
@@ -2440,11 +2747,11 @@
       <c r="F49" s="4"/>
     </row>
     <row r="50" spans="1:6">
-      <c r="A50" s="15" t="s">
+      <c r="A50" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="B50" s="15"/>
-      <c r="C50" s="15" t="s">
+      <c r="B50" s="14"/>
+      <c r="C50" s="14" t="s">
         <v>131</v>
       </c>
       <c r="D50" s="4"/>
@@ -2452,11 +2759,11 @@
       <c r="F50" s="4"/>
     </row>
     <row r="51" spans="1:6">
-      <c r="A51" s="15" t="s">
+      <c r="A51" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="B51" s="15"/>
-      <c r="C51" s="15" t="s">
+      <c r="B51" s="14"/>
+      <c r="C51" s="14" t="s">
         <v>133</v>
       </c>
       <c r="D51" s="4"/>
@@ -2464,11 +2771,11 @@
       <c r="F51" s="4"/>
     </row>
     <row r="52" spans="1:6">
-      <c r="A52" s="15" t="s">
+      <c r="A52" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="B52" s="15"/>
-      <c r="C52" s="15" t="s">
+      <c r="B52" s="14"/>
+      <c r="C52" s="14" t="s">
         <v>135</v>
       </c>
       <c r="D52" s="4"/>
@@ -2476,31 +2783,31 @@
       <c r="F52" s="4"/>
     </row>
     <row r="53" spans="1:6">
-      <c r="A53" s="15"/>
-      <c r="B53" s="15"/>
-      <c r="C53" s="15"/>
+      <c r="A53" s="14"/>
+      <c r="B53" s="14"/>
+      <c r="C53" s="14"/>
       <c r="D53" s="4"/>
       <c r="E53" s="4"/>
       <c r="F53" s="4"/>
     </row>
     <row r="54" spans="1:6" ht="15">
-      <c r="A54" s="23" t="s">
+      <c r="A54" s="22" t="s">
         <v>136</v>
       </c>
-      <c r="B54" s="23"/>
-      <c r="C54" s="23"/>
+      <c r="B54" s="22"/>
+      <c r="C54" s="22"/>
       <c r="D54" s="4"/>
       <c r="E54" s="4"/>
       <c r="F54" s="4"/>
     </row>
     <row r="55" spans="1:6" ht="15">
-      <c r="A55" s="17" t="s">
+      <c r="A55" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B55" s="17" t="s">
+      <c r="B55" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="C55" s="17" t="s">
+      <c r="C55" s="16" t="s">
         <v>91</v>
       </c>
       <c r="D55" s="4"/>
@@ -2508,11 +2815,11 @@
       <c r="F55" s="4"/>
     </row>
     <row r="56" spans="1:6">
-      <c r="A56" s="15" t="s">
+      <c r="A56" s="14" t="s">
         <v>137</v>
       </c>
-      <c r="B56" s="15"/>
-      <c r="C56" s="15" t="s">
+      <c r="B56" s="14"/>
+      <c r="C56" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D56" s="4"/>
@@ -2520,11 +2827,11 @@
       <c r="F56" s="4"/>
     </row>
     <row r="57" spans="1:6">
-      <c r="A57" s="15" t="s">
+      <c r="A57" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="B57" s="15"/>
-      <c r="C57" s="15" t="s">
+      <c r="B57" s="14"/>
+      <c r="C57" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D57" s="4"/>
@@ -2532,11 +2839,11 @@
       <c r="F57" s="4"/>
     </row>
     <row r="58" spans="1:6">
-      <c r="A58" s="15" t="s">
+      <c r="A58" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="B58" s="15"/>
-      <c r="C58" s="15" t="s">
+      <c r="B58" s="14"/>
+      <c r="C58" s="14" t="s">
         <v>105</v>
       </c>
       <c r="D58" s="4"/>
@@ -2544,11 +2851,11 @@
       <c r="F58" s="4"/>
     </row>
     <row r="59" spans="1:6">
-      <c r="A59" s="15" t="s">
+      <c r="A59" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15" t="s">
+      <c r="B59" s="14"/>
+      <c r="C59" s="14" t="s">
         <v>114</v>
       </c>
       <c r="D59" s="4"/>
@@ -2556,11 +2863,11 @@
       <c r="F59" s="4"/>
     </row>
     <row r="60" spans="1:6">
-      <c r="A60" s="15" t="s">
+      <c r="A60" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="B60" s="15"/>
-      <c r="C60" s="15" t="s">
+      <c r="B60" s="14"/>
+      <c r="C60" s="14" t="s">
         <v>142</v>
       </c>
       <c r="D60" s="4"/>
@@ -2568,11 +2875,11 @@
       <c r="F60" s="4"/>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="15" t="s">
+      <c r="A61" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="B61" s="15"/>
-      <c r="C61" s="15" t="s">
+      <c r="B61" s="14"/>
+      <c r="C61" s="14" t="s">
         <v>142</v>
       </c>
       <c r="D61" s="4"/>
@@ -2580,31 +2887,31 @@
       <c r="F61" s="4"/>
     </row>
     <row r="62" spans="1:6">
-      <c r="A62" s="15"/>
-      <c r="B62" s="15"/>
-      <c r="C62" s="15"/>
+      <c r="A62" s="14"/>
+      <c r="B62" s="14"/>
+      <c r="C62" s="14"/>
       <c r="D62" s="4"/>
       <c r="E62" s="4"/>
       <c r="F62" s="4"/>
     </row>
     <row r="63" spans="1:6" ht="15">
-      <c r="A63" s="23" t="s">
+      <c r="A63" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="B63" s="23"/>
-      <c r="C63" s="23"/>
+      <c r="B63" s="22"/>
+      <c r="C63" s="22"/>
       <c r="D63" s="4"/>
       <c r="E63" s="4"/>
       <c r="F63" s="4"/>
     </row>
     <row r="64" spans="1:6" ht="15">
-      <c r="A64" s="17" t="s">
+      <c r="A64" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="B64" s="17" t="s">
+      <c r="B64" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="C64" s="17" t="s">
+      <c r="C64" s="16" t="s">
         <v>91</v>
       </c>
       <c r="D64" s="4"/>
@@ -2612,11 +2919,11 @@
       <c r="F64" s="4"/>
     </row>
     <row r="65" spans="1:6">
-      <c r="A65" s="15" t="s">
+      <c r="A65" s="14" t="s">
         <v>145</v>
       </c>
-      <c r="B65" s="15"/>
-      <c r="C65" s="15" t="s">
+      <c r="B65" s="14"/>
+      <c r="C65" s="14" t="s">
         <v>142</v>
       </c>
       <c r="D65" s="4"/>
@@ -2624,11 +2931,11 @@
       <c r="F65" s="4"/>
     </row>
     <row r="66" spans="1:6">
-      <c r="A66" s="15" t="s">
+      <c r="A66" s="14" t="s">
         <v>146</v>
       </c>
-      <c r="B66" s="15"/>
-      <c r="C66" s="15" t="s">
+      <c r="B66" s="14"/>
+      <c r="C66" s="14" t="s">
         <v>142</v>
       </c>
       <c r="D66" s="4"/>
@@ -2636,11 +2943,11 @@
       <c r="F66" s="4"/>
     </row>
     <row r="67" spans="1:6">
-      <c r="A67" s="15" t="s">
+      <c r="A67" s="14" t="s">
         <v>147</v>
       </c>
-      <c r="B67" s="15"/>
-      <c r="C67" s="15" t="s">
+      <c r="B67" s="14"/>
+      <c r="C67" s="14" t="s">
         <v>142</v>
       </c>
       <c r="D67" s="4"/>
@@ -2648,11 +2955,11 @@
       <c r="F67" s="4"/>
     </row>
     <row r="68" spans="1:6">
-      <c r="A68" s="15" t="s">
+      <c r="A68" s="14" t="s">
         <v>148</v>
       </c>
-      <c r="B68" s="15"/>
-      <c r="C68" s="15" t="s">
+      <c r="B68" s="14"/>
+      <c r="C68" s="14" t="s">
         <v>142</v>
       </c>
       <c r="D68" s="4"/>
@@ -2660,89 +2967,89 @@
       <c r="F68" s="4"/>
     </row>
     <row r="69" spans="1:6">
-      <c r="A69" s="15"/>
-      <c r="B69" s="15"/>
-      <c r="C69" s="15"/>
+      <c r="A69" s="14"/>
+      <c r="B69" s="14"/>
+      <c r="C69" s="14"/>
       <c r="D69" s="4"/>
       <c r="E69" s="4"/>
       <c r="F69" s="4"/>
     </row>
     <row r="70" spans="1:6">
-      <c r="A70" s="15"/>
-      <c r="B70" s="15"/>
-      <c r="C70" s="15"/>
+      <c r="A70" s="14"/>
+      <c r="B70" s="14"/>
+      <c r="C70" s="14"/>
       <c r="D70" s="4"/>
       <c r="E70" s="4"/>
       <c r="F70" s="4"/>
     </row>
     <row r="71" spans="1:6">
-      <c r="A71" s="15"/>
-      <c r="B71" s="15"/>
-      <c r="C71" s="15"/>
+      <c r="A71" s="14"/>
+      <c r="B71" s="14"/>
+      <c r="C71" s="14"/>
       <c r="D71" s="4"/>
       <c r="E71" s="4"/>
       <c r="F71" s="4"/>
     </row>
     <row r="72" spans="1:6">
-      <c r="A72" s="15"/>
-      <c r="B72" s="15"/>
-      <c r="C72" s="15"/>
+      <c r="A72" s="14"/>
+      <c r="B72" s="14"/>
+      <c r="C72" s="14"/>
       <c r="D72" s="4"/>
       <c r="E72" s="4"/>
       <c r="F72" s="4"/>
     </row>
     <row r="73" spans="1:6">
-      <c r="A73" s="15"/>
-      <c r="B73" s="15"/>
-      <c r="C73" s="15"/>
+      <c r="A73" s="14"/>
+      <c r="B73" s="14"/>
+      <c r="C73" s="14"/>
       <c r="D73" s="4"/>
       <c r="E73" s="4"/>
       <c r="F73" s="4"/>
     </row>
     <row r="74" spans="1:6">
-      <c r="A74" s="15"/>
-      <c r="B74" s="15"/>
-      <c r="C74" s="15"/>
+      <c r="A74" s="14"/>
+      <c r="B74" s="14"/>
+      <c r="C74" s="14"/>
       <c r="D74" s="4"/>
       <c r="E74" s="4"/>
       <c r="F74" s="4"/>
     </row>
     <row r="75" spans="1:6">
-      <c r="A75" s="15"/>
-      <c r="B75" s="15"/>
-      <c r="C75" s="15"/>
+      <c r="A75" s="14"/>
+      <c r="B75" s="14"/>
+      <c r="C75" s="14"/>
       <c r="D75" s="4"/>
       <c r="E75" s="4"/>
       <c r="F75" s="4"/>
     </row>
     <row r="76" spans="1:6">
-      <c r="A76" s="15"/>
-      <c r="B76" s="15"/>
-      <c r="C76" s="15"/>
+      <c r="A76" s="14"/>
+      <c r="B76" s="14"/>
+      <c r="C76" s="14"/>
       <c r="D76" s="4"/>
       <c r="E76" s="4"/>
       <c r="F76" s="4"/>
     </row>
     <row r="77" spans="1:6">
-      <c r="A77" s="15"/>
-      <c r="B77" s="15"/>
-      <c r="C77" s="15"/>
+      <c r="A77" s="14"/>
+      <c r="B77" s="14"/>
+      <c r="C77" s="14"/>
       <c r="D77" s="4"/>
       <c r="E77" s="4"/>
       <c r="F77" s="4"/>
     </row>
     <row r="78" spans="1:6">
-      <c r="A78" s="15"/>
-      <c r="B78" s="15"/>
-      <c r="C78" s="15"/>
+      <c r="A78" s="14"/>
+      <c r="B78" s="14"/>
+      <c r="C78" s="14"/>
       <c r="D78" s="4"/>
       <c r="E78" s="4"/>
       <c r="F78" s="4"/>
     </row>
     <row r="79" spans="1:6">
-      <c r="A79" s="15"/>
-      <c r="B79" s="15"/>
-      <c r="C79" s="15"/>
+      <c r="A79" s="14"/>
+      <c r="B79" s="14"/>
+      <c r="C79" s="14"/>
       <c r="D79" s="4"/>
       <c r="E79" s="4"/>
       <c r="F79" s="4"/>
@@ -2777,19 +3084,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22"/>
-      <c r="H1" s="22"/>
-      <c r="I1" s="22"/>
-      <c r="J1" s="22"/>
-      <c r="K1" s="22"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="3" spans="1:11" ht="30">
       <c r="A3" s="5" t="s">
@@ -3505,46 +3812,46 @@
       <c r="N8" s="4"/>
     </row>
     <row r="9" spans="1:14" ht="30">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="15" t="s">
         <v>182</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="15" t="s">
         <v>198</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="15" t="s">
         <v>199</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="15" t="s">
         <v>200</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="15" t="s">
         <v>201</v>
       </c>
-      <c r="F9" s="16" t="s">
+      <c r="F9" s="15" t="s">
         <v>202</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="15" t="s">
         <v>203</v>
       </c>
-      <c r="H9" s="16" t="s">
+      <c r="H9" s="15" t="s">
         <v>204</v>
       </c>
-      <c r="I9" s="16" t="s">
+      <c r="I9" s="15" t="s">
         <v>205</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="J9" s="15" t="s">
         <v>206</v>
       </c>
-      <c r="K9" s="18" t="s">
+      <c r="K9" s="17" t="s">
         <v>207</v>
       </c>
-      <c r="L9" s="18" t="s">
+      <c r="L9" s="17" t="s">
         <v>208</v>
       </c>
-      <c r="M9" s="18" t="s">
+      <c r="M9" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="N9" s="18" t="s">
+      <c r="N9" s="17" t="s">
         <v>210</v>
       </c>
     </row>
@@ -6753,7 +7060,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="144">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="18" t="s">
         <v>236</v>
       </c>
     </row>
@@ -6870,7 +7177,7 @@
       <c r="N7" s="4"/>
     </row>
     <row r="8" spans="1:14" ht="90">
-      <c r="A8" s="20" t="s">
+      <c r="A8" s="19" t="s">
         <v>244</v>
       </c>
     </row>
@@ -6979,7 +7286,7 @@
       <c r="N11" s="4"/>
     </row>
     <row r="12" spans="1:14" ht="105">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="19" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7412,7 +7719,7 @@
       <c r="N23" s="4"/>
     </row>
     <row r="24" spans="1:14" ht="60">
-      <c r="A24" s="20" t="s">
+      <c r="A24" s="19" t="s">
         <v>291</v>
       </c>
     </row>
@@ -7553,7 +7860,7 @@
       <c r="N30" s="4"/>
     </row>
     <row r="31" spans="1:14" ht="45">
-      <c r="A31" s="20" t="s">
+      <c r="A31" s="19" t="s">
         <v>311</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor: remove non-degradable override from Excel contract
</commit_message>
<xml_diff>
--- a/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
+++ b/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ENM\Programming\Repositories\software_BioPot-Gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A6604A-F043-4A60-AA53-82B6643EB78C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1AD74D-B8C8-43E4-94B2-993DBCA1491F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24" yWindow="-12528" windowWidth="22296" windowHeight="11904" firstSheet="4" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_INFORMATIVO" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="353">
   <si>
     <t>BioPot-Gas v0.6 | Informativo do template</t>
   </si>
@@ -146,24 +146,12 @@
     <t>Fração do carbono direcionada à formação de biogás</t>
   </si>
   <si>
-    <t>validate_non_negative</t>
-  </si>
-  <si>
     <t>TRUE</t>
   </si>
   <si>
-    <t>Bloqueia resultados fisicamente inconsistentes</t>
-  </si>
-  <si>
-    <t>include_non_degradable</t>
-  </si>
-  <si>
     <t>FALSE</t>
   </si>
   <si>
-    <t>TRUE inclui não degradáveis no cálculo</t>
-  </si>
-  <si>
     <t>normal_temperature_C</t>
   </si>
   <si>
@@ -191,9 +179,6 @@
     <t>Unidades principais do relatório</t>
   </si>
   <si>
-    <t>Nota: linhas WATER/H2O representam água disponível no sistema, não substrato orgânico. A água é tratada separadamente no balanço de H2O.</t>
-  </si>
-  <si>
     <t>Tabela de componentes, substratos e água disponível</t>
   </si>
   <si>
@@ -317,9 +302,6 @@
     <t>fraction</t>
   </si>
   <si>
-    <t>boolean</t>
-  </si>
-  <si>
     <t>°C</t>
   </si>
   <si>
@@ -1080,6 +1062,48 @@
   </si>
   <si>
     <t>Esta aba não altera o núcleo computacional. Ela organiza evidências de validação e comparação com literatura.</t>
+  </si>
+  <si>
+    <t>Notas: 
+- linhas WATER/H2O representam água disponível no sistema, não substrato orgânico. A água é tratada separadamente no balanço de H2O;
+- degradable = TRUE  → entra no cálculo de BMP;
+- degradable = FALSE → não entra no cálculo de BMP;</t>
+  </si>
+  <si>
+    <t>Componentes não degradáveis</t>
+  </si>
+  <si>
+    <t>Componentes marcados como degradable = FALSE não contribuem para a geração teórica de biogás no cálculo principal de BMP.</t>
+  </si>
+  <si>
+    <t>O core ignora esses componentes antes da soma elementar usada na equação de Buswell.</t>
+  </si>
+  <si>
+    <t>Esta marcação não representa degradação parcial, cinética de degradação ou fração lentamente biodegradável; é uma exclusão estequiométrica binária.</t>
+  </si>
+  <si>
+    <t>Carbono não convertido</t>
+  </si>
+  <si>
+    <t>inert_carbon_mol representa a fração de carbono degradável que não foi direcionada à formação de biogás por carbon_conversion.</t>
+  </si>
+  <si>
+    <t>Calculado como carbono degradável total multiplicado por 1 - carbon_conversion.</t>
+  </si>
+  <si>
+    <t>Não inclui automaticamente o carbono de componentes marcados como degradable = FALSE.</t>
+  </si>
+  <si>
+    <t>Validação de não negatividade</t>
+  </si>
+  <si>
+    <t>Vazões molares, composições elementares e resultados fisicamente inválidos não devem assumir valores negativos no fluxo padrão.</t>
+  </si>
+  <si>
+    <t>O core rejeita vazões molares negativas, carbon_conversion fora de 0 a 1 e composições que levem a resultados fisicamente inconsistentes.</t>
+  </si>
+  <si>
+    <t>Esta validação é uma regra interna do modelo e não pode ser desativada pela aba 01_INPUTS.</t>
   </si>
 </sst>
 </file>
@@ -1247,30 +1271,7 @@
     <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="1" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1291,6 +1292,31 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1467,16 +1493,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
     </row>
     <row r="3" spans="1:8" ht="29.25">
       <c r="A3" s="1" t="s">
@@ -1507,7 +1533,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29.25">
@@ -1552,7 +1578,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N37"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" style="7" customWidth="1"/>
@@ -1567,30 +1593,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
     </row>
     <row r="3" spans="1:14" ht="15">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
     </row>
     <row r="4" spans="1:14" ht="45">
       <c r="A4" s="3" t="s">
@@ -1662,26 +1688,26 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="72">
+    <row r="9" spans="1:14" ht="43.5">
       <c r="A9" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
+      </c>
+      <c r="B9" s="5">
+        <v>0</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="57.75">
+    <row r="10" spans="1:14" ht="29.25">
       <c r="A10" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" s="5" t="s">
         <v>38</v>
+      </c>
+      <c r="B10" s="5">
+        <v>101.325</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>39</v>
@@ -1692,159 +1718,205 @@
     </row>
     <row r="11" spans="1:14" ht="43.5">
       <c r="A11" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B11" s="5">
+        <v>42</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="62.25" customHeight="1">
+      <c r="A14" s="34" t="s">
+        <v>340</v>
+      </c>
+      <c r="B14" s="34"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="34"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="34"/>
+      <c r="G14" s="34"/>
+      <c r="H14" s="34"/>
+      <c r="I14" s="34"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="34"/>
+    </row>
+    <row r="15" spans="1:14" ht="15">
+      <c r="A15" s="27" t="s">
+        <v>45</v>
+      </c>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+    </row>
+    <row r="16" spans="1:14" ht="30">
+      <c r="A16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" s="15" customFormat="1" ht="28.5">
+      <c r="A17" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>306</v>
+      </c>
+      <c r="C17" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="29.25">
-      <c r="A12" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B12" s="5">
-        <v>101.325</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="D12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" ht="43.5">
-      <c r="A13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="D13" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14">
-      <c r="A16" s="18" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="15">
-      <c r="A17" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
-      <c r="M17" s="20"/>
-      <c r="N17" s="20"/>
-    </row>
-    <row r="18" spans="1:14" ht="30">
-      <c r="A18" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="J18" s="3" t="s">
+      <c r="D17" s="16">
+        <v>0</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>307</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16" t="s">
+        <v>305</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>75</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>308</v>
+      </c>
+      <c r="N17" s="17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="B18" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="L18" s="3" t="s">
+      <c r="C18" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D18" s="6">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="M18" s="3" t="s">
+      <c r="L18" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="N18" s="3" t="s">
+      <c r="M18" s="6" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="19" spans="1:14" s="15" customFormat="1" ht="28.5">
-      <c r="A19" s="16" t="s">
-        <v>311</v>
-      </c>
-      <c r="B19" s="16" t="s">
-        <v>312</v>
-      </c>
-      <c r="C19" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="D19" s="16">
-        <v>0</v>
-      </c>
-      <c r="E19" s="16" t="s">
-        <v>313</v>
-      </c>
-      <c r="F19" s="16"/>
-      <c r="G19" s="16"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16" t="s">
-        <v>311</v>
-      </c>
-      <c r="L19" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="M19" s="16" t="s">
-        <v>314</v>
-      </c>
-      <c r="N19" s="17" t="b">
-        <v>1</v>
+      <c r="N18" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14">
+      <c r="A19" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="6">
+        <v>0.5</v>
+      </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+      <c r="K19" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="L19" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M19" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N19" s="6" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D20" s="6">
-        <v>1</v>
+        <v>0.2</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -1853,30 +1925,30 @@
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="L20" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="N20" s="6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="28.5">
+      <c r="A21" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M20" s="6" t="s">
+      <c r="B21" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="N20" s="6" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14">
-      <c r="A21" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="C21" s="6" t="s">
         <v>35</v>
       </c>
       <c r="D21" s="6">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -1885,16 +1957,16 @@
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -1905,373 +1977,310 @@
         <v>72</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D22" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="E22" s="6"/>
+        <v>0</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="N22" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="28.5">
+    <row r="23" spans="1:14">
       <c r="A23" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D23" s="6">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="6"/>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
+      <c r="F23" s="6">
+        <v>6</v>
+      </c>
+      <c r="G23" s="6">
+        <v>10</v>
+      </c>
+      <c r="H23" s="6">
+        <v>5</v>
+      </c>
+      <c r="I23" s="6">
+        <v>0</v>
+      </c>
+      <c r="J23" s="6">
+        <v>0</v>
+      </c>
       <c r="K23" s="6" t="s">
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="L23" s="6" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N23" s="6" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:14">
-      <c r="A24" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D24" s="6">
-        <v>0</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="F24" s="6"/>
-      <c r="G24" s="6"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
-      <c r="K24" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="M24" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="N24" s="6" t="s">
-        <v>38</v>
-      </c>
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18"/>
+      <c r="L24" s="18"/>
+      <c r="M24" s="18"/>
+      <c r="N24" s="18"/>
     </row>
     <row r="25" spans="1:14">
-      <c r="A25" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="B25" s="6" t="s">
-        <v>77</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D25" s="6">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6">
-        <v>6</v>
-      </c>
-      <c r="G25" s="6">
-        <v>10</v>
-      </c>
-      <c r="H25" s="6">
-        <v>5</v>
-      </c>
-      <c r="I25" s="6">
-        <v>0</v>
-      </c>
-      <c r="J25" s="6">
-        <v>0</v>
-      </c>
-      <c r="K25" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="L25" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="M25" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="N25" s="6" t="s">
-        <v>38</v>
-      </c>
+      <c r="A25" s="18"/>
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="18"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18"/>
+      <c r="L25" s="18"/>
+      <c r="M25" s="18"/>
+      <c r="N25" s="18"/>
     </row>
     <row r="26" spans="1:14">
-      <c r="A26" s="19"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="19"/>
-      <c r="J26" s="19"/>
-      <c r="K26" s="19"/>
-      <c r="L26" s="19"/>
-      <c r="M26" s="19"/>
-      <c r="N26" s="19"/>
+      <c r="A26" s="18"/>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
+      <c r="L26" s="18"/>
+      <c r="M26" s="18"/>
+      <c r="N26" s="18"/>
     </row>
     <row r="27" spans="1:14">
-      <c r="A27" s="19"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="19"/>
-      <c r="J27" s="19"/>
-      <c r="K27" s="19"/>
-      <c r="L27" s="19"/>
-      <c r="M27" s="19"/>
-      <c r="N27" s="19"/>
+      <c r="A27" s="18"/>
+      <c r="B27" s="18"/>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="18"/>
+      <c r="M27" s="18"/>
+      <c r="N27" s="18"/>
     </row>
     <row r="28" spans="1:14">
-      <c r="A28" s="19"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="19"/>
+      <c r="A28" s="18"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="18"/>
+      <c r="K28" s="18"/>
+      <c r="L28" s="18"/>
+      <c r="M28" s="18"/>
+      <c r="N28" s="18"/>
     </row>
     <row r="29" spans="1:14">
-      <c r="A29" s="19"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="19"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="19"/>
-      <c r="N29" s="19"/>
+      <c r="A29" s="18"/>
+      <c r="B29" s="18"/>
+      <c r="C29" s="18"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
+      <c r="I29" s="18"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="18"/>
+      <c r="L29" s="18"/>
+      <c r="M29" s="18"/>
+      <c r="N29" s="18"/>
     </row>
     <row r="30" spans="1:14">
-      <c r="A30" s="19"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="19"/>
+      <c r="A30" s="18"/>
+      <c r="B30" s="18"/>
+      <c r="C30" s="18"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="18"/>
+      <c r="M30" s="18"/>
+      <c r="N30" s="18"/>
     </row>
     <row r="31" spans="1:14">
-      <c r="A31" s="19"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="19"/>
-      <c r="J31" s="19"/>
-      <c r="K31" s="19"/>
-      <c r="L31" s="19"/>
-      <c r="M31" s="19"/>
-      <c r="N31" s="19"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="18"/>
+      <c r="C31" s="18"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="18"/>
+      <c r="L31" s="18"/>
+      <c r="M31" s="18"/>
+      <c r="N31" s="18"/>
     </row>
     <row r="32" spans="1:14">
-      <c r="A32" s="19"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="19"/>
-      <c r="J32" s="19"/>
-      <c r="K32" s="19"/>
-      <c r="L32" s="19"/>
-      <c r="M32" s="19"/>
-      <c r="N32" s="19"/>
+      <c r="A32" s="18"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
     </row>
     <row r="33" spans="1:14">
-      <c r="A33" s="19"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="19"/>
-      <c r="J33" s="19"/>
-      <c r="K33" s="19"/>
-      <c r="L33" s="19"/>
-      <c r="M33" s="19"/>
-      <c r="N33" s="19"/>
+      <c r="A33" s="18"/>
+      <c r="B33" s="18"/>
+      <c r="C33" s="18"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="18"/>
+      <c r="M33" s="18"/>
+      <c r="N33" s="18"/>
     </row>
     <row r="34" spans="1:14">
-      <c r="A34" s="19"/>
-      <c r="B34" s="19"/>
-      <c r="C34" s="19"/>
-      <c r="D34" s="19"/>
-      <c r="E34" s="19"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="19"/>
-      <c r="J34" s="19"/>
-      <c r="K34" s="19"/>
-      <c r="L34" s="19"/>
-      <c r="M34" s="19"/>
-      <c r="N34" s="19"/>
+      <c r="A34" s="18"/>
+      <c r="B34" s="18"/>
+      <c r="C34" s="18"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="18"/>
+      <c r="L34" s="18"/>
+      <c r="M34" s="18"/>
+      <c r="N34" s="18"/>
     </row>
     <row r="35" spans="1:14">
-      <c r="A35" s="19"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="19"/>
-      <c r="D35" s="19"/>
-      <c r="E35" s="19"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="19"/>
-      <c r="J35" s="19"/>
-      <c r="K35" s="19"/>
-      <c r="L35" s="19"/>
-      <c r="M35" s="19"/>
-      <c r="N35" s="19"/>
+      <c r="A35" s="18"/>
+      <c r="B35" s="18"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="18"/>
+      <c r="L35" s="18"/>
+      <c r="M35" s="18"/>
+      <c r="N35" s="18"/>
     </row>
     <row r="36" spans="1:14">
-      <c r="A36" s="19"/>
-      <c r="B36" s="19"/>
-      <c r="C36" s="19"/>
-      <c r="D36" s="19"/>
-      <c r="E36" s="19"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="19"/>
-      <c r="J36" s="19"/>
-      <c r="K36" s="19"/>
-      <c r="L36" s="19"/>
-      <c r="M36" s="19"/>
-      <c r="N36" s="19"/>
+      <c r="A36" s="18"/>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="18"/>
+      <c r="L36" s="18"/>
+      <c r="M36" s="18"/>
+      <c r="N36" s="18"/>
     </row>
     <row r="37" spans="1:14">
-      <c r="A37" s="19"/>
-      <c r="B37" s="19"/>
-      <c r="C37" s="19"/>
-      <c r="D37" s="19"/>
-      <c r="E37" s="19"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="19"/>
-      <c r="J37" s="19"/>
-      <c r="K37" s="19"/>
-      <c r="L37" s="19"/>
-      <c r="M37" s="19"/>
-      <c r="N37" s="19"/>
-    </row>
-    <row r="38" spans="1:14">
-      <c r="A38" s="19"/>
-      <c r="B38" s="19"/>
-      <c r="C38" s="19"/>
-      <c r="D38" s="19"/>
-      <c r="E38" s="19"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="19"/>
-      <c r="J38" s="19"/>
-      <c r="K38" s="19"/>
-      <c r="L38" s="19"/>
-      <c r="M38" s="19"/>
-      <c r="N38" s="19"/>
-    </row>
-    <row r="39" spans="1:14">
-      <c r="A39" s="19"/>
-      <c r="B39" s="19"/>
-      <c r="C39" s="19"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="19"/>
-      <c r="J39" s="19"/>
-      <c r="K39" s="19"/>
-      <c r="L39" s="19"/>
-      <c r="M39" s="19"/>
-      <c r="N39" s="19"/>
+      <c r="A37" s="18"/>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
+      <c r="J37" s="18"/>
+      <c r="K37" s="18"/>
+      <c r="L37" s="18"/>
+      <c r="M37" s="18"/>
+      <c r="N37" s="18"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A17:N17"/>
+  <mergeCells count="4">
+    <mergeCell ref="A15:N15"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A14:K14"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="C20:C199 N20:N199" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" sqref="C18:C197 N18:N197" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="K20:K199" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="K18:K197" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"DATABASE,FORMULA,ELEMENTS"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2281,7 +2290,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F78"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="34" style="7" customWidth="1"/>
@@ -2291,28 +2300,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1">
-      <c r="A1" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
+      <c r="A1" s="29" t="s">
+        <v>79</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
     </row>
     <row r="2" spans="1:6" ht="15">
-      <c r="A2" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
+      <c r="A2" s="28" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="28"/>
+      <c r="C2" s="28"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="13" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -2379,21 +2388,21 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15">
-      <c r="A9" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
+      <c r="A9" s="28" t="s">
+        <v>84</v>
+      </c>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="13" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -2405,7 +2414,7 @@
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -2413,11 +2422,11 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -2425,11 +2434,11 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="12" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2437,86 +2446,86 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="12" t="s">
-        <v>42</v>
+        <v>88</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+      <c r="A15" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>96</v>
-      </c>
+        <v>91</v>
+      </c>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>97</v>
+      <c r="A17" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12" t="s">
+        <v>93</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="12" t="s">
-        <v>98</v>
-      </c>
+      <c r="A18" s="12"/>
       <c r="B18" s="12"/>
-      <c r="C18" s="12" t="s">
-        <v>99</v>
-      </c>
+      <c r="C18" s="12"/>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
+    <row r="19" spans="1:6" ht="15">
+      <c r="A19" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" ht="15">
-      <c r="A20" s="23" t="s">
-        <v>100</v>
-      </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
+      <c r="A20" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="1:6" ht="15">
-      <c r="A21" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B21" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C21" s="14" t="s">
-        <v>88</v>
+    <row r="21" spans="1:6">
+      <c r="A21" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12" t="s">
+        <v>96</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -2524,11 +2533,11 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="12" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
@@ -2536,11 +2545,11 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="12" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -2548,86 +2557,86 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="12" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="12" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
+      <c r="A25" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="7" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C26" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="12" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="27" spans="1:6">
-      <c r="A27" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>90</v>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12" t="s">
+        <v>96</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="12" t="s">
-        <v>108</v>
-      </c>
+      <c r="A28" s="12"/>
       <c r="B28" s="12"/>
-      <c r="C28" s="12" t="s">
-        <v>102</v>
-      </c>
+      <c r="C28" s="12"/>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="1:6">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
+    <row r="29" spans="1:6" ht="15">
+      <c r="A29" s="30" t="s">
+        <v>103</v>
+      </c>
+      <c r="B29" s="30"/>
+      <c r="C29" s="30"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="15">
-      <c r="A30" s="23" t="s">
-        <v>109</v>
-      </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="23"/>
+      <c r="A30" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B30" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="31" spans="1:6" ht="15">
-      <c r="A31" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B31" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C31" s="14" t="s">
-        <v>88</v>
+    <row r="31" spans="1:6">
+      <c r="A31" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12" t="s">
+        <v>105</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -2635,23 +2644,22 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="12" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12" t="s">
-        <v>111</v>
+      <c r="A33" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>105</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -2659,91 +2667,91 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="7" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
+        <v>105</v>
+      </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="7" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>111</v>
-      </c>
+        <v>105</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="7" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>111</v>
-      </c>
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
       <c r="D37" s="2"/>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
     </row>
-    <row r="38" spans="1:6">
-      <c r="A38" s="12"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
+    <row r="38" spans="1:6" s="7" customFormat="1" ht="15">
+      <c r="A38" s="30" t="s">
+        <v>111</v>
+      </c>
+      <c r="B38" s="30"/>
+      <c r="C38" s="30"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
-    <row r="39" spans="1:6" s="7" customFormat="1" ht="15">
-      <c r="A39" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="B39" s="23"/>
-      <c r="C39" s="23"/>
+    <row r="39" spans="1:6" ht="15">
+      <c r="A39" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B39" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
     </row>
-    <row r="40" spans="1:6" ht="15">
-      <c r="A40" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B40" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C40" s="14" t="s">
-        <v>88</v>
-      </c>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
+    <row r="40" spans="1:6">
+      <c r="A40" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="7" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>119</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="7" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2751,21 +2759,22 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="7" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
     </row>
     <row r="44" spans="1:6">
-      <c r="A44" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="C44" s="7" t="s">
-        <v>119</v>
+      <c r="A44" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="B44" s="12"/>
+      <c r="C44" s="12" t="s">
+        <v>113</v>
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
@@ -2773,7 +2782,7 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="12" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="12" t="s">
@@ -2784,44 +2793,44 @@
       <c r="F45" s="2"/>
     </row>
     <row r="46" spans="1:6">
-      <c r="A46" s="12" t="s">
-        <v>124</v>
-      </c>
+      <c r="A46" s="12"/>
       <c r="B46" s="12"/>
-      <c r="C46" s="12" t="s">
-        <v>125</v>
-      </c>
+      <c r="C46" s="12"/>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
     </row>
-    <row r="47" spans="1:6">
-      <c r="A47" s="12"/>
-      <c r="B47" s="12"/>
-      <c r="C47" s="12"/>
+    <row r="47" spans="1:6" ht="15">
+      <c r="A47" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="B47" s="30"/>
+      <c r="C47" s="30"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
     </row>
     <row r="48" spans="1:6" ht="15">
-      <c r="A48" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="B48" s="23"/>
-      <c r="C48" s="23"/>
+      <c r="A48" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B48" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C48" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
       <c r="F48" s="2"/>
     </row>
-    <row r="49" spans="1:6" ht="15">
-      <c r="A49" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B49" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C49" s="14" t="s">
-        <v>88</v>
+    <row r="49" spans="1:6">
+      <c r="A49" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="B49" s="12"/>
+      <c r="C49" s="12" t="s">
+        <v>122</v>
       </c>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
@@ -2829,11 +2838,11 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="12" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="12" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
@@ -2841,55 +2850,55 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="12" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="12" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
     </row>
     <row r="52" spans="1:6">
-      <c r="A52" s="12" t="s">
-        <v>131</v>
-      </c>
+      <c r="A52" s="12"/>
       <c r="B52" s="12"/>
-      <c r="C52" s="12" t="s">
-        <v>132</v>
-      </c>
+      <c r="C52" s="12"/>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
       <c r="F52" s="2"/>
     </row>
-    <row r="53" spans="1:6">
-      <c r="A53" s="12"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="12"/>
+    <row r="53" spans="1:6" ht="15">
+      <c r="A53" s="30" t="s">
+        <v>127</v>
+      </c>
+      <c r="B53" s="30"/>
+      <c r="C53" s="30"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
     </row>
     <row r="54" spans="1:6" ht="15">
-      <c r="A54" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="B54" s="23"/>
-      <c r="C54" s="23"/>
+      <c r="A54" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B54" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C54" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
       <c r="F54" s="2"/>
     </row>
-    <row r="55" spans="1:6" ht="15">
-      <c r="A55" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B55" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C55" s="14" t="s">
-        <v>88</v>
+    <row r="55" spans="1:6">
+      <c r="A55" s="12" t="s">
+        <v>128</v>
+      </c>
+      <c r="B55" s="12"/>
+      <c r="C55" s="12" t="s">
+        <v>96</v>
       </c>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
@@ -2897,11 +2906,11 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="12" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B56" s="12"/>
       <c r="C56" s="12" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
@@ -2909,11 +2918,11 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="12" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="12" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
@@ -2921,11 +2930,11 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="12" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B58" s="12"/>
       <c r="C58" s="12" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
@@ -2933,11 +2942,11 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="12" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="12" t="s">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -2945,55 +2954,55 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="12" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="B60" s="12"/>
       <c r="C60" s="12" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
     </row>
     <row r="61" spans="1:6">
-      <c r="A61" s="12" t="s">
-        <v>140</v>
-      </c>
+      <c r="A61" s="12"/>
       <c r="B61" s="12"/>
-      <c r="C61" s="12" t="s">
-        <v>139</v>
-      </c>
+      <c r="C61" s="12"/>
       <c r="D61" s="2"/>
       <c r="E61" s="2"/>
       <c r="F61" s="2"/>
     </row>
-    <row r="62" spans="1:6">
-      <c r="A62" s="12"/>
-      <c r="B62" s="12"/>
-      <c r="C62" s="12"/>
+    <row r="62" spans="1:6" ht="15">
+      <c r="A62" s="30" t="s">
+        <v>135</v>
+      </c>
+      <c r="B62" s="30"/>
+      <c r="C62" s="30"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
     </row>
     <row r="63" spans="1:6" ht="15">
-      <c r="A63" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="B63" s="23"/>
-      <c r="C63" s="23"/>
+      <c r="A63" s="14" t="s">
+        <v>81</v>
+      </c>
+      <c r="B63" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="C63" s="14" t="s">
+        <v>83</v>
+      </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
       <c r="F63" s="2"/>
     </row>
-    <row r="64" spans="1:6" ht="15">
-      <c r="A64" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="B64" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C64" s="14" t="s">
-        <v>88</v>
+    <row r="64" spans="1:6">
+      <c r="A64" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="B64" s="12"/>
+      <c r="C64" s="12" t="s">
+        <v>133</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
@@ -3001,11 +3010,11 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="12" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="12" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
@@ -3013,11 +3022,11 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="12" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="12" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -3025,24 +3034,20 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="12" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="12" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
       <c r="F67" s="2"/>
     </row>
     <row r="68" spans="1:6">
-      <c r="A68" s="12" t="s">
-        <v>145</v>
-      </c>
+      <c r="A68" s="12"/>
       <c r="B68" s="12"/>
-      <c r="C68" s="12" t="s">
-        <v>139</v>
-      </c>
+      <c r="C68" s="12"/>
       <c r="D68" s="2"/>
       <c r="E68" s="2"/>
       <c r="F68" s="2"/>
@@ -3127,25 +3132,17 @@
       <c r="E78" s="2"/>
       <c r="F78" s="2"/>
     </row>
-    <row r="79" spans="1:6">
-      <c r="A79" s="12"/>
-      <c r="B79" s="12"/>
-      <c r="C79" s="12"/>
-      <c r="D79" s="2"/>
-      <c r="E79" s="2"/>
-      <c r="F79" s="2"/>
-    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A63:C63"/>
-    <mergeCell ref="A54:C54"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A62:C62"/>
+    <mergeCell ref="A53:C53"/>
+    <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A19:C19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3165,61 +3162,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18">
-      <c r="A1" s="24" t="s">
-        <v>146</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
+      <c r="A1" s="26" t="s">
+        <v>140</v>
+      </c>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="31"/>
+      <c r="H1" s="31"/>
+      <c r="I1" s="31"/>
+      <c r="J1" s="31"/>
+      <c r="K1" s="31"/>
     </row>
     <row r="3" spans="1:11" ht="30">
       <c r="A3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="H3" s="3" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C4" s="2">
         <v>6</v>
@@ -3237,24 +3234,24 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="C5" s="2">
         <v>12</v>
@@ -3272,24 +3269,24 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C6" s="2">
         <v>5</v>
@@ -3307,24 +3304,24 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C7" s="2">
         <v>6</v>
@@ -3342,24 +3339,24 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C8" s="2">
         <v>5</v>
@@ -3377,24 +3374,24 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C9" s="2">
         <v>6</v>
@@ -3412,24 +3409,24 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
@@ -3447,24 +3444,24 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
@@ -3482,24 +3479,24 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C12" s="2">
         <v>5</v>
@@ -3517,24 +3514,24 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="2" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
@@ -3552,24 +3549,24 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C14" s="2">
         <v>5</v>
@@ -3587,24 +3584,24 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C15" s="2">
         <v>3</v>
@@ -3622,24 +3619,24 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -3657,24 +3654,24 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="C17" s="2">
         <v>7.3</v>
@@ -3692,24 +3689,24 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -3727,16 +3724,16 @@
         <v>3.5000000000000001E-3</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -3761,70 +3758,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18">
-      <c r="A1" s="24" t="s">
-        <v>178</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24"/>
-      <c r="I1" s="24"/>
-      <c r="J1" s="24"/>
-      <c r="K1" s="24"/>
-      <c r="L1" s="24"/>
-      <c r="M1" s="24"/>
-      <c r="N1" s="24"/>
+      <c r="A1" s="26" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="26"/>
+      <c r="I1" s="26"/>
+      <c r="J1" s="26"/>
+      <c r="K1" s="26"/>
+      <c r="L1" s="26"/>
+      <c r="M1" s="26"/>
+      <c r="N1" s="26"/>
     </row>
     <row r="3" spans="1:14" ht="30">
       <c r="A3" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>181</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>182</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>183</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>190</v>
-      </c>
       <c r="M3" s="3" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3838,15 +3835,15 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -3861,7 +3858,7 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -3897,65 +3894,65 @@
       <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="15">
-      <c r="A8" s="20" t="s">
-        <v>194</v>
-      </c>
-      <c r="B8" s="20"/>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="20"/>
-      <c r="J8" s="20"/>
-      <c r="K8" s="20"/>
-      <c r="L8" s="20"/>
-      <c r="M8" s="20"/>
-      <c r="N8" s="20"/>
+      <c r="A8" s="27" t="s">
+        <v>188</v>
+      </c>
+      <c r="B8" s="27"/>
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
+      <c r="L8" s="27"/>
+      <c r="M8" s="27"/>
+      <c r="N8" s="27"/>
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="13" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="B9" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="H9" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>203</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>206</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -7030,7 +7027,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" style="7" customWidth="1"/>
@@ -7039,67 +7036,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18">
-      <c r="A1" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
+      <c r="A1" s="26" t="s">
+        <v>202</v>
+      </c>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="3" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="B4" s="30" t="s">
-        <v>331</v>
+        <v>207</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>325</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28.5">
       <c r="A5" s="2" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="57">
       <c r="A6" s="2" t="s">
-        <v>220</v>
-      </c>
-      <c r="B6" s="29" t="s">
-        <v>342</v>
-      </c>
-      <c r="C6" s="33" t="s">
-        <v>343</v>
+        <v>214</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>336</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>337</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -7107,125 +7104,167 @@
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="31" t="s">
-        <v>332</v>
-      </c>
-      <c r="C8" s="31" t="s">
-        <v>333</v>
-      </c>
-      <c r="D8" s="31" t="s">
-        <v>226</v>
+      <c r="B8" s="22" t="s">
+        <v>326</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="15" customFormat="1" ht="57">
-      <c r="A9" s="28" t="s">
-        <v>334</v>
+      <c r="A9" s="19" t="s">
+        <v>328</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28.5">
       <c r="A10" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="B10" s="32" t="s">
-        <v>336</v>
-      </c>
-      <c r="C10" s="32" t="s">
-        <v>337</v>
+        <v>221</v>
+      </c>
+      <c r="B10" s="23" t="s">
+        <v>330</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>331</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A11" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>340</v>
+        <v>334</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="42.75">
       <c r="A12" s="2" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="42.75">
       <c r="A13" s="2" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="28.5">
       <c r="A14" s="2" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42.75">
       <c r="A15" s="2" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>330</v>
+        <v>324</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="42.75">
+      <c r="A16" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>343</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="28.5">
+      <c r="A17" s="2" t="s">
+        <v>345</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="42.75">
+      <c r="A18" s="2" t="s">
+        <v>349</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>350</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -7257,22 +7296,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18">
-      <c r="A1" s="27" t="s">
-        <v>229</v>
-      </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
-      <c r="K1" s="27"/>
-      <c r="L1" s="27"/>
-      <c r="M1" s="27"/>
-      <c r="N1" s="27"/>
+      <c r="A1" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
+      <c r="M1" s="33"/>
+      <c r="N1" s="33"/>
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="2"/>
@@ -7295,7 +7334,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -7312,10 +7351,10 @@
     </row>
     <row r="4" spans="1:14" ht="57.75">
       <c r="A4" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="B4" s="34" t="s">
-        <v>345</v>
+        <v>225</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>339</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -7332,10 +7371,10 @@
     </row>
     <row r="5" spans="1:14" ht="114.75">
       <c r="A5" s="10" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -7352,10 +7391,10 @@
     </row>
     <row r="6" spans="1:14" ht="29.25">
       <c r="A6" s="10" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -7387,79 +7426,79 @@
       <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="15">
-      <c r="A8" s="26" t="s">
-        <v>236</v>
-      </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="26"/>
-      <c r="L8" s="26"/>
-      <c r="M8" s="26"/>
-      <c r="N8" s="26"/>
+      <c r="A8" s="32" t="s">
+        <v>230</v>
+      </c>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="32"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+      <c r="K8" s="32"/>
+      <c r="L8" s="32"/>
+      <c r="M8" s="32"/>
+      <c r="N8" s="32"/>
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="11" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>32</v>
       </c>
       <c r="F9" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="L9" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>243</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>244</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>245</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>246</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>247</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="85.5">
       <c r="A10" s="8" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="E10" s="8">
         <v>1</v>
@@ -7486,10 +7525,10 @@
         <v>-6.9879518072294089E-2</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -7509,79 +7548,79 @@
       <c r="N11" s="2"/>
     </row>
     <row r="12" spans="1:14" ht="15">
-      <c r="A12" s="26" t="s">
-        <v>255</v>
-      </c>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="26"/>
-      <c r="F12" s="26"/>
-      <c r="G12" s="26"/>
-      <c r="H12" s="26"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="26"/>
-      <c r="K12" s="26"/>
-      <c r="L12" s="26"/>
-      <c r="M12" s="26"/>
-      <c r="N12" s="26"/>
+      <c r="A12" s="32" t="s">
+        <v>249</v>
+      </c>
+      <c r="B12" s="32"/>
+      <c r="C12" s="32"/>
+      <c r="D12" s="32"/>
+      <c r="E12" s="32"/>
+      <c r="F12" s="32"/>
+      <c r="G12" s="32"/>
+      <c r="H12" s="32"/>
+      <c r="I12" s="32"/>
+      <c r="J12" s="32"/>
+      <c r="K12" s="32"/>
+      <c r="L12" s="32"/>
+      <c r="M12" s="32"/>
+      <c r="N12" s="32"/>
     </row>
     <row r="13" spans="1:14" ht="30">
       <c r="A13" s="11" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="D13" s="11" t="s">
+        <v>250</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>251</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>253</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>254</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>255</v>
+      </c>
+      <c r="J13" s="11" t="s">
         <v>256</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="K13" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>257</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="N13" s="11" t="s">
         <v>258</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>259</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>260</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>261</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>262</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>263</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="28.5">
       <c r="A14" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="E14" s="8">
         <v>490.11</v>
@@ -7602,30 +7641,30 @@
         <v>-8.4128576014130138E-2</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L14" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M14" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="28.5">
       <c r="A15" s="8" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C15" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>267</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>273</v>
       </c>
       <c r="E15" s="8">
         <v>490.11</v>
@@ -7646,30 +7685,30 @@
         <v>-0.1649644901525206</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M15" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.5">
       <c r="A16" s="8" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="E16" s="8">
         <v>428.4</v>
@@ -7690,30 +7729,30 @@
         <v>1.6132982587243029E-2</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M16" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.5">
       <c r="A17" s="8" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="E17" s="8">
         <v>428.4</v>
@@ -7734,30 +7773,30 @@
         <v>8.7237397338995933E-3</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M17" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N17" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.5">
       <c r="A18" s="8" t="s">
-        <v>277</v>
+        <v>271</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="E18" s="8">
         <v>484.63</v>
@@ -7778,30 +7817,30 @@
         <v>-4.5187050999701966E-3</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L18" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M18" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N18" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.5">
       <c r="A19" s="8" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="E19" s="8">
         <v>484.63</v>
@@ -7822,30 +7861,30 @@
         <v>-4.0114456608485519E-3</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.5">
       <c r="A20" s="8" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="E20" s="8">
         <v>413.02</v>
@@ -7866,30 +7905,30 @@
         <v>-6.0227292075755966E-3</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M20" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.5">
       <c r="A21" s="8" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="E21" s="8">
         <v>413.02</v>
@@ -7910,16 +7949,16 @@
         <v>4.72329903258944E-4</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="M21" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="N21" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -7955,29 +7994,29 @@
       <c r="N23" s="2"/>
     </row>
     <row r="24" spans="1:14" ht="15">
-      <c r="A24" s="26" t="s">
-        <v>283</v>
-      </c>
-      <c r="B24" s="26"/>
-      <c r="C24" s="26"/>
-      <c r="D24" s="26"/>
-      <c r="E24" s="26"/>
+      <c r="A24" s="32" t="s">
+        <v>277</v>
+      </c>
+      <c r="B24" s="32"/>
+      <c r="C24" s="32"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="32"/>
     </row>
     <row r="25" spans="1:14" ht="30">
       <c r="A25" s="11" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -7991,19 +8030,19 @@
     </row>
     <row r="26" spans="1:14" ht="85.5">
       <c r="A26" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -8017,19 +8056,19 @@
     </row>
     <row r="27" spans="1:14" ht="85.5">
       <c r="A27" s="9" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>297</v>
+        <v>291</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -8043,19 +8082,19 @@
     </row>
     <row r="28" spans="1:14" ht="71.25">
       <c r="A28" s="9" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -8100,17 +8139,17 @@
       <c r="N30" s="2"/>
     </row>
     <row r="31" spans="1:14" ht="15">
-      <c r="A31" s="26" t="s">
-        <v>303</v>
-      </c>
-      <c r="B31" s="26"/>
+      <c r="A31" s="32" t="s">
+        <v>297</v>
+      </c>
+      <c r="B31" s="32"/>
     </row>
     <row r="32" spans="1:14" ht="15">
       <c r="A32" s="11" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -8127,10 +8166,10 @@
     </row>
     <row r="33" spans="1:14" ht="57">
       <c r="A33" s="2" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -8147,10 +8186,10 @@
     </row>
     <row r="34" spans="1:14" ht="57">
       <c r="A34" s="2" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -8167,10 +8206,10 @@
     </row>
     <row r="35" spans="1:14" ht="42.75">
       <c r="A35" s="2" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -8187,10 +8226,10 @@
     </row>
     <row r="36" spans="1:14" ht="57">
       <c r="A36" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -8207,10 +8246,10 @@
     </row>
     <row r="37" spans="1:14" ht="57">
       <c r="A37" s="2" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>

</xml_diff>

<commit_message>
feat: support molar and mass Excel input bases
</commit_message>
<xml_diff>
--- a/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
+++ b/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ENM\Programming\Repositories\software_BioPot-Gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C1AD74D-B8C8-43E4-94B2-993DBCA1491F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A74D88-36A6-4FC4-97C5-E672C9471C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24" yWindow="-12528" windowWidth="22296" windowHeight="11904" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_INFORMATIVO" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,10 @@
     <sheet name="05_METHOD_NOTES" sheetId="6" r:id="rId6"/>
     <sheet name="06_VALIDATION_BENCHMARKS" sheetId="7" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="mass">'01_INPUTS'!$AC$4:$AC$9</definedName>
+    <definedName name="molar">'01_INPUTS'!$AB$4:$AB$7</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -42,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="573" uniqueCount="353">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="361">
   <si>
     <t>BioPot-Gas v0.6 | Informativo do template</t>
   </si>
@@ -191,9 +195,6 @@
     <t>degradable</t>
   </si>
   <si>
-    <t>molar_flow</t>
-  </si>
-  <si>
     <t>formula</t>
   </si>
   <si>
@@ -332,9 +333,6 @@
     <t>CH4_mol</t>
   </si>
   <si>
-    <t>input molar basis</t>
-  </si>
-  <si>
     <t>CO2_mol</t>
   </si>
   <si>
@@ -359,9 +357,6 @@
     <t>CH4_mass</t>
   </si>
   <si>
-    <t>kg if input basis is kmol</t>
-  </si>
-  <si>
     <t>CO2_mass</t>
   </si>
   <si>
@@ -383,9 +378,6 @@
     <t>CH4_Nm3</t>
   </si>
   <si>
-    <t>Nm³</t>
-  </si>
-  <si>
     <t>CO2_Nm3</t>
   </si>
   <si>
@@ -410,13 +402,7 @@
     <t>CH4_energy_LHV_MJ</t>
   </si>
   <si>
-    <t>MJ</t>
-  </si>
-  <si>
     <t>CH4_energy_LHV_kWh</t>
-  </si>
-  <si>
-    <t>kWh</t>
   </si>
   <si>
     <t>CH4_to_CO2_molar_ratio</t>
@@ -1104,6 +1090,48 @@
   </si>
   <si>
     <t>Esta validação é uma regra interna do modelo e não pode ser desativada pela aba 01_INPUTS.</t>
+  </si>
+  <si>
+    <t>mol</t>
+  </si>
+  <si>
+    <t>kmol</t>
+  </si>
+  <si>
+    <t>mol/h</t>
+  </si>
+  <si>
+    <t>input_basis_type</t>
+  </si>
+  <si>
+    <t>input_unit</t>
+  </si>
+  <si>
+    <t>input_quantity</t>
+  </si>
+  <si>
+    <t>mass</t>
+  </si>
+  <si>
+    <t>molar</t>
+  </si>
+  <si>
+    <t>kg</t>
+  </si>
+  <si>
+    <t>g</t>
+  </si>
+  <si>
+    <t>ton</t>
+  </si>
+  <si>
+    <t>kg/h</t>
+  </si>
+  <si>
+    <t>ton/h</t>
+  </si>
+  <si>
+    <t>g/h</t>
   </si>
 </sst>
 </file>
@@ -1226,7 +1254,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1299,6 +1327,9 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -1315,9 +1346,9 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1533,7 +1564,7 @@
         <v>7</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>338</v>
+        <v>332</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29.25">
@@ -1578,12 +1609,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N37"/>
+  <dimension ref="A1:AC38"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" style="7" customWidth="1"/>
     <col min="2" max="2" width="18" style="7" customWidth="1"/>
-    <col min="3" max="4" width="12" style="7" customWidth="1"/>
+    <col min="3" max="3" width="12" style="7" customWidth="1"/>
+    <col min="4" max="4" width="13.75" style="7" customWidth="1"/>
     <col min="5" max="5" width="24" style="7" customWidth="1"/>
     <col min="6" max="10" width="10" style="7" customWidth="1"/>
     <col min="11" max="11" width="14" style="7" customWidth="1"/>
@@ -1592,7 +1624,7 @@
     <col min="14" max="14" width="12" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18">
+    <row r="1" spans="1:29" ht="18">
       <c r="A1" s="26" t="s">
         <v>16</v>
       </c>
@@ -1610,15 +1642,24 @@
       <c r="M1" s="26"/>
       <c r="N1" s="26"/>
     </row>
-    <row r="3" spans="1:14" ht="15">
+    <row r="3" spans="1:29" ht="15">
       <c r="A3" s="27" t="s">
         <v>17</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
       <c r="D3" s="27"/>
-    </row>
-    <row r="4" spans="1:14" ht="45">
+      <c r="AA3" t="s">
+        <v>350</v>
+      </c>
+      <c r="AB3" t="s">
+        <v>354</v>
+      </c>
+      <c r="AC3" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="4" spans="1:29" ht="45">
       <c r="A4" s="3" t="s">
         <v>18</v>
       </c>
@@ -1631,8 +1672,17 @@
       <c r="D4" s="3" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" ht="57.75">
+      <c r="AA4" t="s">
+        <v>354</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>347</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="5" spans="1:29" ht="57.75">
       <c r="A5" s="4" t="s">
         <v>22</v>
       </c>
@@ -1645,8 +1695,17 @@
       <c r="D5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="43.5">
+      <c r="AA5" t="s">
+        <v>353</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>348</v>
+      </c>
+      <c r="AC5" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="6" spans="1:29" ht="43.5">
       <c r="A6" s="4" t="s">
         <v>26</v>
       </c>
@@ -1659,232 +1718,228 @@
       <c r="D6" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" ht="129">
-      <c r="A7" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="AB6" t="s">
+        <v>349</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" s="15" customFormat="1" ht="15">
+      <c r="A7" s="35" t="s">
+        <v>350</v>
+      </c>
+      <c r="B7" s="36" t="s">
+        <v>354</v>
+      </c>
+      <c r="C7" s="19"/>
+      <c r="AB7" t="s">
         <v>30</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="AC7" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="8" spans="1:29" ht="129">
+      <c r="A8" s="4" t="s">
+        <v>351</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>31</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" ht="72">
-      <c r="A8" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B8" s="5">
-        <v>0.95</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>33</v>
       </c>
       <c r="D8" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" ht="43.5">
+      <c r="AB8" s="15"/>
+      <c r="AC8" s="15" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="9" spans="1:29" ht="72">
       <c r="A9" s="4" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="B9" s="5">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" ht="29.25">
+      <c r="AC9" s="37" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="10" spans="1:29" ht="43.5">
       <c r="A10" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B10" s="5">
-        <v>101.325</v>
+        <v>0</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="43.5">
+    <row r="11" spans="1:29" ht="29.25">
       <c r="A11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B11" s="5">
+        <v>101.325</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D11" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:29" ht="43.5">
+      <c r="A12" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B12" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D12" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="14" spans="1:14" ht="62.25" customHeight="1">
-      <c r="A14" s="34" t="s">
-        <v>340</v>
-      </c>
-      <c r="B14" s="34"/>
-      <c r="C14" s="34"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="34"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="34"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="34"/>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-    </row>
-    <row r="15" spans="1:14" ht="15">
-      <c r="A15" s="27" t="s">
+    <row r="15" spans="1:29" ht="62.25" customHeight="1">
+      <c r="A15" s="28" t="s">
+        <v>334</v>
+      </c>
+      <c r="B15" s="28"/>
+      <c r="C15" s="28"/>
+      <c r="D15" s="28"/>
+      <c r="E15" s="28"/>
+      <c r="F15" s="28"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="28"/>
+      <c r="I15" s="28"/>
+      <c r="J15" s="28"/>
+      <c r="K15" s="28"/>
+    </row>
+    <row r="16" spans="1:29" ht="15">
+      <c r="A16" s="27" t="s">
         <v>45</v>
       </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
-    </row>
-    <row r="16" spans="1:14" ht="30">
-      <c r="A16" s="3" t="s">
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
+    </row>
+    <row r="17" spans="1:14" ht="15">
+      <c r="A17" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="D17" s="3" t="s">
+        <v>352</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H17" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="I17" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="J17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="K17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="L17" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="M17" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="N17" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="N16" s="3" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" s="15" customFormat="1" ht="28.5">
-      <c r="A17" s="16" t="s">
-        <v>305</v>
-      </c>
-      <c r="B17" s="16" t="s">
-        <v>306</v>
-      </c>
-      <c r="C17" s="17" t="b">
+    </row>
+    <row r="18" spans="1:14" s="15" customFormat="1" ht="28.5">
+      <c r="A18" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="B18" s="16" t="s">
+        <v>300</v>
+      </c>
+      <c r="C18" s="17" t="b">
         <v>0</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D18" s="16">
         <v>0</v>
       </c>
-      <c r="E17" s="16" t="s">
-        <v>307</v>
-      </c>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16" t="s">
-        <v>305</v>
-      </c>
-      <c r="L17" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="M17" s="16" t="s">
-        <v>308</v>
-      </c>
-      <c r="N17" s="17" t="b">
+      <c r="E18" s="16" t="s">
+        <v>301</v>
+      </c>
+      <c r="F18" s="16"/>
+      <c r="G18" s="16"/>
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16" t="s">
+        <v>299</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>302</v>
+      </c>
+      <c r="N18" s="17" t="b">
         <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14">
-      <c r="A18" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D18" s="6">
-        <v>1</v>
-      </c>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
-      <c r="K18" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="L18" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="M18" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="N18" s="6" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="6" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C19" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D19" s="6">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
@@ -1893,13 +1948,13 @@
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="L19" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="M19" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="M19" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="N19" s="6" t="s">
         <v>34</v>
@@ -1907,16 +1962,16 @@
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C20" s="6" t="s">
         <v>34</v>
       </c>
       <c r="D20" s="6">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -1925,30 +1980,30 @@
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="L20" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="M20" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="M20" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="N20" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="28.5">
+    <row r="21" spans="1:14">
       <c r="A21" s="6" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D21" s="6">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -1957,58 +2012,56 @@
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="M21" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="M21" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="N21" s="6" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" ht="28.5">
       <c r="A22" s="6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D22" s="6">
-        <v>0</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>73</v>
-      </c>
+        <v>0.1</v>
+      </c>
+      <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="6" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C23" s="6" t="s">
         <v>34</v>
@@ -2016,50 +2069,68 @@
       <c r="D23" s="6">
         <v>0</v>
       </c>
-      <c r="E23" s="6"/>
-      <c r="F23" s="6">
-        <v>6</v>
-      </c>
-      <c r="G23" s="6">
-        <v>10</v>
-      </c>
-      <c r="H23" s="6">
-        <v>5</v>
-      </c>
-      <c r="I23" s="6">
-        <v>0</v>
-      </c>
-      <c r="J23" s="6">
-        <v>0</v>
-      </c>
+      <c r="E23" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
+      <c r="J23" s="6"/>
       <c r="K23" s="6" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="L23" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M23" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="M23" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="N23" s="6" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:14">
-      <c r="A24" s="18"/>
-      <c r="B24" s="18"/>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="18"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="18"/>
-      <c r="N24" s="18"/>
+      <c r="A24" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="6">
+        <v>0</v>
+      </c>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6">
+        <v>6</v>
+      </c>
+      <c r="G24" s="6">
+        <v>10</v>
+      </c>
+      <c r="H24" s="6">
+        <v>5</v>
+      </c>
+      <c r="I24" s="6">
+        <v>0</v>
+      </c>
+      <c r="J24" s="6">
+        <v>0</v>
+      </c>
+      <c r="K24" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="L24" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="M24" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="N24" s="6" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="18"/>
@@ -2269,19 +2340,41 @@
       <c r="M37" s="18"/>
       <c r="N37" s="18"/>
     </row>
+    <row r="38" spans="1:14">
+      <c r="A38" s="18"/>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="18"/>
+      <c r="J38" s="18"/>
+      <c r="K38" s="18"/>
+      <c r="L38" s="18"/>
+      <c r="M38" s="18"/>
+      <c r="N38" s="18"/>
+    </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A15:N15"/>
+    <mergeCell ref="A16:N16"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A15:K15"/>
   </mergeCells>
-  <dataValidations count="2">
-    <dataValidation type="list" sqref="C18:C197 N18:N197" xr:uid="{00000000-0002-0000-0100-000000000000}">
+  <dataValidations count="4">
+    <dataValidation type="list" sqref="C19:C198 N19:N198" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="K18:K197" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="K19:K198" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"DATABASE,FORMULA,ELEMENTS"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{A6C2391F-5F62-4932-8555-2C756A0F9999}">
+      <formula1>INDIRECT($B$7)</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7" xr:uid="{22E2C124-66E9-4DF6-803E-F15A91FD1CEE}">
+      <formula1>$AA$4:$AA$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2300,28 +2393,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1">
-      <c r="A1" s="29" t="s">
+      <c r="A1" s="30" t="s">
+        <v>78</v>
+      </c>
+      <c r="B1" s="30"/>
+      <c r="C1" s="30"/>
+    </row>
+    <row r="2" spans="1:6" ht="15">
+      <c r="A2" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="29"/>
-      <c r="C1" s="29"/>
-    </row>
-    <row r="2" spans="1:6" ht="15">
-      <c r="A2" s="28" t="s">
-        <v>80</v>
-      </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C3" s="13" t="s">
         <v>82</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>83</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -2371,7 +2464,7 @@
         <v>29</v>
       </c>
       <c r="B7" s="12" t="str">
-        <f>'01_INPUTS'!B7</f>
+        <f>'01_INPUTS'!B8</f>
         <v>kmol/h</v>
       </c>
       <c r="C7" s="12"/>
@@ -2388,21 +2481,21 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15">
-      <c r="A9" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="28"/>
-      <c r="C9" s="28"/>
+      <c r="A9" s="29" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="13" t="s">
         <v>82</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>83</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -2414,7 +2507,7 @@
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -2426,7 +2519,7 @@
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -2438,7 +2531,7 @@
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2446,11 +2539,11 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -2461,7 +2554,7 @@
         <v>40</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2469,7 +2562,7 @@
         <v>41</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -2477,11 +2570,11 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -2496,24 +2589,24 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="15">
-      <c r="A19" s="30" t="s">
-        <v>94</v>
-      </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
+      <c r="A19" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="B19" s="31"/>
+      <c r="C19" s="31"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" ht="15">
       <c r="A20" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="C20" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -2521,66 +2614,55 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B21" s="12"/>
-      <c r="C21" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C21" s="12"/>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="12" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B22" s="12"/>
-      <c r="C22" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C22" s="12"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="12" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B23" s="12"/>
-      <c r="C23" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C23" s="12"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="12" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B24" s="12"/>
-      <c r="C24" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C24" s="12"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -2588,12 +2670,10 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="12" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B27" s="12"/>
-      <c r="C27" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C27" s="12"/>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -2607,24 +2687,24 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="15">
-      <c r="A29" s="30" t="s">
-        <v>103</v>
-      </c>
-      <c r="B29" s="30"/>
-      <c r="C29" s="30"/>
+      <c r="A29" s="31" t="s">
+        <v>101</v>
+      </c>
+      <c r="B29" s="31"/>
+      <c r="C29" s="31"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="15">
       <c r="A30" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="C30" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -2632,34 +2712,27 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="12" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B31" s="12"/>
-      <c r="C31" s="12" t="s">
-        <v>105</v>
-      </c>
+      <c r="C31" s="12"/>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="12" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B32" s="12"/>
-      <c r="C32" s="12" t="s">
-        <v>105</v>
-      </c>
+      <c r="C32" s="12"/>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="7" t="s">
-        <v>107</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -2667,18 +2740,12 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C34" s="7" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="C35" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -2686,10 +2753,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C36" s="7" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -2704,24 +2768,24 @@
       <c r="F37" s="2"/>
     </row>
     <row r="38" spans="1:6" s="7" customFormat="1" ht="15">
-      <c r="A38" s="30" t="s">
-        <v>111</v>
-      </c>
-      <c r="B38" s="30"/>
-      <c r="C38" s="30"/>
+      <c r="A38" s="31" t="s">
+        <v>108</v>
+      </c>
+      <c r="B38" s="31"/>
+      <c r="C38" s="31"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
     <row r="39" spans="1:6" ht="15">
       <c r="A39" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B39" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="C39" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -2729,18 +2793,12 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="C40" s="7" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C41" s="7" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -2748,10 +2806,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="C42" s="7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2759,10 +2814,7 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C43" s="7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -2770,23 +2822,21 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="12" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B44" s="12"/>
-      <c r="C44" s="12" t="s">
-        <v>113</v>
-      </c>
+      <c r="C44" s="12"/>
       <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="12" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -2801,24 +2851,24 @@
       <c r="F46" s="2"/>
     </row>
     <row r="47" spans="1:6" ht="15">
-      <c r="A47" s="30" t="s">
-        <v>120</v>
-      </c>
-      <c r="B47" s="30"/>
-      <c r="C47" s="30"/>
+      <c r="A47" s="31" t="s">
+        <v>116</v>
+      </c>
+      <c r="B47" s="31"/>
+      <c r="C47" s="31"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
     </row>
     <row r="48" spans="1:6" ht="15">
       <c r="A48" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B48" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B48" s="14" t="s">
+      <c r="C48" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="C48" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
@@ -2826,35 +2876,31 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="12" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B49" s="12"/>
-      <c r="C49" s="12" t="s">
-        <v>122</v>
-      </c>
+      <c r="C49" s="12"/>
       <c r="D49" s="2"/>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="12" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B50" s="12"/>
-      <c r="C50" s="12" t="s">
-        <v>124</v>
-      </c>
+      <c r="C50" s="12"/>
       <c r="D50" s="2"/>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="12" t="s">
-        <v>125</v>
+        <v>119</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="12" t="s">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
@@ -2869,24 +2915,24 @@
       <c r="F52" s="2"/>
     </row>
     <row r="53" spans="1:6" ht="15">
-      <c r="A53" s="30" t="s">
-        <v>127</v>
-      </c>
-      <c r="B53" s="30"/>
-      <c r="C53" s="30"/>
+      <c r="A53" s="31" t="s">
+        <v>121</v>
+      </c>
+      <c r="B53" s="31"/>
+      <c r="C53" s="31"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
     </row>
     <row r="54" spans="1:6" ht="15">
       <c r="A54" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B54" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B54" s="14" t="s">
+      <c r="C54" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -2894,59 +2940,51 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="12" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B55" s="12"/>
-      <c r="C55" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C55" s="12"/>
       <c r="D55" s="2"/>
       <c r="E55" s="2"/>
       <c r="F55" s="2"/>
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="12" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="B56" s="12"/>
-      <c r="C56" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C56" s="12"/>
       <c r="D56" s="2"/>
       <c r="E56" s="2"/>
       <c r="F56" s="2"/>
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="12" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="B57" s="12"/>
-      <c r="C57" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="C57" s="12"/>
       <c r="D57" s="2"/>
       <c r="E57" s="2"/>
       <c r="F57" s="2"/>
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="12" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="B58" s="12"/>
-      <c r="C58" s="12" t="s">
-        <v>105</v>
-      </c>
+      <c r="C58" s="12"/>
       <c r="D58" s="2"/>
       <c r="E58" s="2"/>
       <c r="F58" s="2"/>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="12" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -2954,11 +2992,11 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="12" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B60" s="12"/>
       <c r="C60" s="12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -2973,24 +3011,24 @@
       <c r="F61" s="2"/>
     </row>
     <row r="62" spans="1:6" ht="15">
-      <c r="A62" s="30" t="s">
-        <v>135</v>
-      </c>
-      <c r="B62" s="30"/>
-      <c r="C62" s="30"/>
+      <c r="A62" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="B62" s="31"/>
+      <c r="C62" s="31"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
     </row>
     <row r="63" spans="1:6" ht="15">
       <c r="A63" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B63" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="B63" s="14" t="s">
+      <c r="C63" s="14" t="s">
         <v>82</v>
-      </c>
-      <c r="C63" s="14" t="s">
-        <v>83</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
@@ -2998,11 +3036,11 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="12" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B64" s="12"/>
       <c r="C64" s="12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
@@ -3010,11 +3048,11 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="12" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
@@ -3022,11 +3060,11 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="12" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -3034,11 +3072,11 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="12" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="12" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
@@ -3163,60 +3201,60 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18">
       <c r="A1" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="31"/>
-      <c r="I1" s="31"/>
-      <c r="J1" s="31"/>
-      <c r="K1" s="31"/>
+        <v>134</v>
+      </c>
+      <c r="B1" s="32"/>
+      <c r="C1" s="32"/>
+      <c r="D1" s="32"/>
+      <c r="E1" s="32"/>
+      <c r="F1" s="32"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="32"/>
+      <c r="I1" s="32"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="32"/>
     </row>
     <row r="3" spans="1:11" ht="30">
       <c r="A3" s="3" t="s">
         <v>46</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>47</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C4" s="2">
         <v>6</v>
@@ -3234,13 +3272,13 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K4" s="2" t="s">
         <v>34</v>
@@ -3248,10 +3286,10 @@
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C5" s="2">
         <v>12</v>
@@ -3269,13 +3307,13 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K5" s="2" t="s">
         <v>34</v>
@@ -3283,10 +3321,10 @@
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C6" s="2">
         <v>5</v>
@@ -3304,13 +3342,13 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K6" s="2" t="s">
         <v>34</v>
@@ -3318,10 +3356,10 @@
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="C7" s="2">
         <v>6</v>
@@ -3339,13 +3377,13 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K7" s="2" t="s">
         <v>34</v>
@@ -3353,10 +3391,10 @@
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C8" s="2">
         <v>5</v>
@@ -3374,13 +3412,13 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K8" s="2" t="s">
         <v>34</v>
@@ -3388,10 +3426,10 @@
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="2" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C9" s="2">
         <v>6</v>
@@ -3409,13 +3447,13 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K9" s="2" t="s">
         <v>34</v>
@@ -3423,10 +3461,10 @@
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="2" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
@@ -3444,13 +3482,13 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K10" s="2" t="s">
         <v>34</v>
@@ -3458,10 +3496,10 @@
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
@@ -3479,13 +3517,13 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K11" s="2" t="s">
         <v>34</v>
@@ -3493,10 +3531,10 @@
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="2" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C12" s="2">
         <v>5</v>
@@ -3514,13 +3552,13 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>34</v>
@@ -3528,10 +3566,10 @@
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="2" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
@@ -3549,13 +3587,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K13" s="2" t="s">
         <v>34</v>
@@ -3563,10 +3601,10 @@
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="2" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C14" s="2">
         <v>5</v>
@@ -3584,13 +3622,13 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K14" s="2" t="s">
         <v>34</v>
@@ -3598,10 +3636,10 @@
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C15" s="2">
         <v>3</v>
@@ -3619,13 +3657,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K15" s="2" t="s">
         <v>34</v>
@@ -3633,10 +3671,10 @@
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -3654,13 +3692,13 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>34</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K16" s="2" t="s">
         <v>34</v>
@@ -3668,10 +3706,10 @@
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="C17" s="2">
         <v>7.3</v>
@@ -3689,13 +3727,13 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>35</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>34</v>
@@ -3703,10 +3741,10 @@
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="2" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -3724,13 +3762,13 @@
         <v>3.5000000000000001E-3</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>35</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="K18" s="2" t="s">
         <v>34</v>
@@ -3759,7 +3797,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18">
       <c r="A1" s="26" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -3777,51 +3815,51 @@
     </row>
     <row r="3" spans="1:14" ht="30">
       <c r="A3" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>184</v>
-      </c>
       <c r="M3" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3835,7 +3873,7 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="N4" s="2" t="s">
         <v>34</v>
@@ -3843,7 +3881,7 @@
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -3895,7 +3933,7 @@
     </row>
     <row r="8" spans="1:14" ht="15">
       <c r="A8" s="27" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="B8" s="27"/>
       <c r="C8" s="27"/>
@@ -3913,46 +3951,46 @@
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="13" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B9" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="H9" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>195</v>
-      </c>
-      <c r="I9" s="13" t="s">
-        <v>196</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>197</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>198</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>200</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -7037,7 +7075,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18">
       <c r="A1" s="26" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -7045,58 +7083,58 @@
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="3" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>325</v>
+        <v>319</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="28.5">
       <c r="A5" s="2" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="57">
       <c r="A6" s="2" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="B6" s="20" t="s">
-        <v>336</v>
+        <v>330</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>337</v>
+        <v>331</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -7104,13 +7142,13 @@
         <v>10</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -7118,153 +7156,153 @@
         <v>12</v>
       </c>
       <c r="B8" s="22" t="s">
-        <v>326</v>
+        <v>320</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>327</v>
+        <v>321</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A9" s="19" t="s">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>329</v>
+        <v>323</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="28.5">
       <c r="A10" s="2" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="B10" s="23" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="C10" s="23" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A11" t="s">
-        <v>335</v>
+        <v>329</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>332</v>
+        <v>326</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>333</v>
+        <v>327</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>334</v>
+        <v>328</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="42.75">
       <c r="A12" s="2" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>311</v>
+        <v>305</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>312</v>
+        <v>306</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="42.75">
       <c r="A13" s="2" t="s">
-        <v>313</v>
+        <v>307</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>314</v>
+        <v>308</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>315</v>
+        <v>309</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>316</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="28.5">
       <c r="A14" s="2" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>319</v>
+        <v>313</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>320</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="42.75">
       <c r="A15" s="2" t="s">
-        <v>321</v>
+        <v>315</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>322</v>
+        <v>316</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>323</v>
+        <v>317</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="42.75">
       <c r="A16" s="2" t="s">
-        <v>341</v>
+        <v>335</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>342</v>
+        <v>336</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>343</v>
+        <v>337</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>344</v>
+        <v>338</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="28.5">
       <c r="A17" s="2" t="s">
-        <v>345</v>
+        <v>339</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>346</v>
+        <v>340</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>347</v>
+        <v>341</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="42.75">
       <c r="A18" s="2" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>352</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>
@@ -7296,22 +7334,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18">
-      <c r="A1" s="33" t="s">
-        <v>223</v>
-      </c>
-      <c r="B1" s="33"/>
-      <c r="C1" s="33"/>
-      <c r="D1" s="33"/>
-      <c r="E1" s="33"/>
-      <c r="F1" s="33"/>
-      <c r="G1" s="33"/>
-      <c r="H1" s="33"/>
-      <c r="I1" s="33"/>
-      <c r="J1" s="33"/>
-      <c r="K1" s="33"/>
-      <c r="L1" s="33"/>
-      <c r="M1" s="33"/>
-      <c r="N1" s="33"/>
+      <c r="A1" s="34" t="s">
+        <v>217</v>
+      </c>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="34"/>
+      <c r="N1" s="34"/>
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="2"/>
@@ -7334,7 +7372,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -7351,10 +7389,10 @@
     </row>
     <row r="4" spans="1:14" ht="57.75">
       <c r="A4" s="10" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>339</v>
+        <v>333</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -7371,10 +7409,10 @@
     </row>
     <row r="5" spans="1:14" ht="114.75">
       <c r="A5" s="10" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -7391,10 +7429,10 @@
     </row>
     <row r="6" spans="1:14" ht="29.25">
       <c r="A6" s="10" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -7426,79 +7464,79 @@
       <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="15">
-      <c r="A8" s="32" t="s">
-        <v>230</v>
-      </c>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="32"/>
-      <c r="L8" s="32"/>
-      <c r="M8" s="32"/>
-      <c r="N8" s="32"/>
+      <c r="A8" s="33" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8" s="33"/>
+      <c r="C8" s="33"/>
+      <c r="D8" s="33"/>
+      <c r="E8" s="33"/>
+      <c r="F8" s="33"/>
+      <c r="G8" s="33"/>
+      <c r="H8" s="33"/>
+      <c r="I8" s="33"/>
+      <c r="J8" s="33"/>
+      <c r="K8" s="33"/>
+      <c r="L8" s="33"/>
+      <c r="M8" s="33"/>
+      <c r="N8" s="33"/>
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="11" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="E9" s="11" t="s">
         <v>32</v>
       </c>
       <c r="F9" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>232</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="L9" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>236</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>237</v>
-      </c>
-      <c r="I9" s="11" t="s">
-        <v>238</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>239</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>241</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="85.5">
       <c r="A10" s="8" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E10" s="8">
         <v>1</v>
@@ -7525,10 +7563,10 @@
         <v>-6.9879518072294089E-2</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -7548,79 +7586,79 @@
       <c r="N11" s="2"/>
     </row>
     <row r="12" spans="1:14" ht="15">
-      <c r="A12" s="32" t="s">
-        <v>249</v>
-      </c>
-      <c r="B12" s="32"/>
-      <c r="C12" s="32"/>
-      <c r="D12" s="32"/>
-      <c r="E12" s="32"/>
-      <c r="F12" s="32"/>
-      <c r="G12" s="32"/>
-      <c r="H12" s="32"/>
-      <c r="I12" s="32"/>
-      <c r="J12" s="32"/>
-      <c r="K12" s="32"/>
-      <c r="L12" s="32"/>
-      <c r="M12" s="32"/>
-      <c r="N12" s="32"/>
+      <c r="A12" s="33" t="s">
+        <v>243</v>
+      </c>
+      <c r="B12" s="33"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="33"/>
+      <c r="E12" s="33"/>
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="33"/>
+      <c r="J12" s="33"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="33"/>
+      <c r="N12" s="33"/>
     </row>
     <row r="13" spans="1:14" ht="30">
       <c r="A13" s="11" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="D13" s="11" t="s">
+        <v>244</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>245</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>246</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="I13" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="J13" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="K13" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>251</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="N13" s="11" t="s">
         <v>252</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>253</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>256</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>242</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>243</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>257</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="28.5">
       <c r="A14" s="8" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="E14" s="8">
         <v>490.11</v>
@@ -7641,30 +7679,30 @@
         <v>-8.4128576014130138E-2</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L14" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M14" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="28.5">
       <c r="A15" s="8" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C15" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>261</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>267</v>
       </c>
       <c r="E15" s="8">
         <v>490.11</v>
@@ -7685,30 +7723,30 @@
         <v>-0.1649644901525206</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M15" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.5">
       <c r="A16" s="8" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="E16" s="8">
         <v>428.4</v>
@@ -7729,30 +7767,30 @@
         <v>1.6132982587243029E-2</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M16" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.5">
       <c r="A17" s="8" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="E17" s="8">
         <v>428.4</v>
@@ -7773,30 +7811,30 @@
         <v>8.7237397338995933E-3</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M17" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N17" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.5">
       <c r="A18" s="8" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="E18" s="8">
         <v>484.63</v>
@@ -7817,30 +7855,30 @@
         <v>-4.5187050999701966E-3</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L18" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M18" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N18" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.5">
       <c r="A19" s="8" t="s">
-        <v>273</v>
+        <v>267</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="E19" s="8">
         <v>484.63</v>
@@ -7861,30 +7899,30 @@
         <v>-4.0114456608485519E-3</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.5">
       <c r="A20" s="8" t="s">
-        <v>274</v>
+        <v>268</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="E20" s="8">
         <v>413.02</v>
@@ -7905,30 +7943,30 @@
         <v>-6.0227292075755966E-3</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M20" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.5">
       <c r="A21" s="8" t="s">
-        <v>276</v>
+        <v>270</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>275</v>
+        <v>269</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="E21" s="8">
         <v>413.02</v>
@@ -7949,16 +7987,16 @@
         <v>4.72329903258944E-4</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M21" s="8" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="N21" s="8" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -7994,29 +8032,29 @@
       <c r="N23" s="2"/>
     </row>
     <row r="24" spans="1:14" ht="15">
-      <c r="A24" s="32" t="s">
-        <v>277</v>
-      </c>
-      <c r="B24" s="32"/>
-      <c r="C24" s="32"/>
-      <c r="D24" s="32"/>
-      <c r="E24" s="32"/>
+      <c r="A24" s="33" t="s">
+        <v>271</v>
+      </c>
+      <c r="B24" s="33"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="33"/>
+      <c r="E24" s="33"/>
     </row>
     <row r="25" spans="1:14" ht="30">
       <c r="A25" s="11" t="s">
-        <v>278</v>
+        <v>272</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>279</v>
+        <v>273</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>281</v>
+        <v>275</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -8030,19 +8068,19 @@
     </row>
     <row r="26" spans="1:14" ht="85.5">
       <c r="A26" s="9" t="s">
-        <v>282</v>
+        <v>276</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>284</v>
+        <v>278</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>285</v>
+        <v>279</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>286</v>
+        <v>280</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -8056,19 +8094,19 @@
     </row>
     <row r="27" spans="1:14" ht="85.5">
       <c r="A27" s="9" t="s">
-        <v>287</v>
+        <v>281</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>288</v>
+        <v>282</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>289</v>
+        <v>283</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>290</v>
+        <v>284</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>291</v>
+        <v>285</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -8082,19 +8120,19 @@
     </row>
     <row r="28" spans="1:14" ht="71.25">
       <c r="A28" s="9" t="s">
-        <v>292</v>
+        <v>286</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>296</v>
+        <v>290</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -8139,17 +8177,17 @@
       <c r="N30" s="2"/>
     </row>
     <row r="31" spans="1:14" ht="15">
-      <c r="A31" s="32" t="s">
-        <v>297</v>
-      </c>
-      <c r="B31" s="32"/>
+      <c r="A31" s="33" t="s">
+        <v>291</v>
+      </c>
+      <c r="B31" s="33"/>
     </row>
     <row r="32" spans="1:14" ht="15">
       <c r="A32" s="11" t="s">
-        <v>298</v>
+        <v>292</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>299</v>
+        <v>293</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -8166,10 +8204,10 @@
     </row>
     <row r="33" spans="1:14" ht="57">
       <c r="A33" s="2" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -8186,10 +8224,10 @@
     </row>
     <row r="34" spans="1:14" ht="57">
       <c r="A34" s="2" t="s">
-        <v>301</v>
+        <v>295</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -8206,10 +8244,10 @@
     </row>
     <row r="35" spans="1:14" ht="42.75">
       <c r="A35" s="2" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -8226,10 +8264,10 @@
     </row>
     <row r="36" spans="1:14" ht="57">
       <c r="A36" s="2" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -8246,10 +8284,10 @@
     </row>
     <row r="37" spans="1:14" ht="57">
       <c r="A37" s="2" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>

</xml_diff>

<commit_message>
docs: document Excel input bases and output units
</commit_message>
<xml_diff>
--- a/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
+++ b/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ENM\Programming\Repositories\software_BioPot-Gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40A74D88-36A6-4FC4-97C5-E672C9471C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22111DD-33CE-4670-AA91-64E70B7CF2DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24" yWindow="-12528" windowWidth="22296" windowHeight="11904" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-24" yWindow="-12528" windowWidth="22296" windowHeight="11904" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_INFORMATIVO" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="381">
   <si>
     <t>BioPot-Gas v0.6 | Informativo do template</t>
   </si>
@@ -69,9 +69,6 @@
     <t>01_INPUTS recebe parâmetros globais e componentes. 02_OUTPUTS recebe resultados automáticos. 03_COMPONENT_DATABASE contém componentes padronizados. 04_EXPERIMENTAL_VALIDATION compara dados experimentais e teóricos. 05_METHOD_NOTES registra hipóteses e limites.</t>
   </si>
   <si>
-    <t>Unidade molar</t>
-  </si>
-  <si>
     <t>Condição normal</t>
   </si>
   <si>
@@ -1017,9 +1014,6 @@
     <t>Fechamento estequimétrico</t>
   </si>
   <si>
-    <t>É necessária manter a consistência entre as bases dos componentes degradáveis com a água declarada presente na composição e/ou na vazão da corrente material.</t>
-  </si>
-  <si>
     <t>A rotina pode funcionar de forma autônoma ou ser integrada a outros ambientes.</t>
   </si>
   <si>
@@ -1042,9 +1036,6 @@
   </si>
   <si>
     <t>T e P podem ser informados na planilha, caso contrário, são utilizados os parâmetros internos R, T e P.</t>
-  </si>
-  <si>
-    <t>Use uma base molar consistente para todos os componentes. Use kmol ou kmol/h para interpretar diretamente as massas em kg e os volumes normalizados em Nm³. O software preserva a base declarada nas saídas molares.</t>
   </si>
   <si>
     <t>Esta aba não altera o núcleo computacional. Ela organiza evidências de validação e comparação com literatura.</t>
@@ -1068,18 +1059,6 @@
     <t>Esta marcação não representa degradação parcial, cinética de degradação ou fração lentamente biodegradável; é uma exclusão estequiométrica binária.</t>
   </si>
   <si>
-    <t>Carbono não convertido</t>
-  </si>
-  <si>
-    <t>inert_carbon_mol representa a fração de carbono degradável que não foi direcionada à formação de biogás por carbon_conversion.</t>
-  </si>
-  <si>
-    <t>Calculado como carbono degradável total multiplicado por 1 - carbon_conversion.</t>
-  </si>
-  <si>
-    <t>Não inclui automaticamente o carbono de componentes marcados como degradable = FALSE.</t>
-  </si>
-  <si>
     <t>Validação de não negatividade</t>
   </si>
   <si>
@@ -1132,6 +1111,87 @@
   </si>
   <si>
     <t>g/h</t>
+  </si>
+  <si>
+    <t>Carbono inerte reportado</t>
+  </si>
+  <si>
+    <t>inert_carbon_mol representa a fração de carbono degradável que não foi convertida segundo carbon_conversion.</t>
+  </si>
+  <si>
+    <t>O valor é calculado apenas a partir dos componentes degradáveis incluídos no cálculo estequiométrico. Componentes marcados como non-degradable/degradable = FALSE são excluídos do cálculo de Buswell e não contribuem para inert_carbon_mol.</t>
+  </si>
+  <si>
+    <t>Este campo não representa todo o carbono fisicamente inerte presente na alimentação. Ele representa apenas o carbono degradável não convertido pelo fator carbon_conversion.</t>
+  </si>
+  <si>
+    <t>Massa de carbono inerte reportado</t>
+  </si>
+  <si>
+    <t>inert_carbon_mass é a conversão mássica de inert_carbon_mol usando a massa atômica do carbono.</t>
+  </si>
+  <si>
+    <t>Como inert_carbon_mol se refere apenas a carbono não convertido em gás, o valor reportado não se refere à massa molecular do substrato original.</t>
+  </si>
+  <si>
+    <t>A unidade de saída é kg para entradas em quantidade e kg/h para entradas em vazão, calculada a partir da massa atômica do carbono.</t>
+  </si>
+  <si>
+    <t>É necessária manter a consistência entre as unidades dos componentes degradáveis com a água declarada.</t>
+  </si>
+  <si>
+    <t>Base global de entrada</t>
+  </si>
+  <si>
+    <t>input_basis_type e input_unit definem a base usada para todos os valores da coluna input_quantity.</t>
+  </si>
+  <si>
+    <t>O template aceita entradas em base molar ou mássica. Em base molar, são aceitas kmol, mol, kmol/h e mol/h. Em base mássica, são aceitas kg, g, ton, kg/h, g/h e ton/h. O pipeline converte todas as entradas para uma base molar interna antes do cálculo estequiométrico.</t>
+  </si>
+  <si>
+    <t>O template não permite misturar unidades diferentes entre linhas da tabela de componentes. A unidade é global para toda a alimentação.</t>
+  </si>
+  <si>
+    <t>Conversão de entrada mássica para base molar</t>
+  </si>
+  <si>
+    <t>A massa informada em input_quantity é convertida para kg e dividida pela massa molar do componente em kg/kmol. O resultado é uma quantidade molar interna usada pelo core.</t>
+  </si>
+  <si>
+    <t>Para linhas WATER/H2O, a conversão usa a massa molecular da água. Componentes sem composição elementar válida não podem ser convertidos corretamente.</t>
+  </si>
+  <si>
+    <t>O programa permite informar os dados de entrada em base mássica em input_basis_type. Quando input_basis_type = mass, o pipeline calcula a massa molar de cada componente a partir da composição elementar C, H, O, N e S.</t>
+  </si>
+  <si>
+    <t>Unidades de saída padronizadas</t>
+  </si>
+  <si>
+    <t>A coluna Unidade em 02_OUTPUTS é preenchida automaticamente pelo writer conforme basis_time_mode.</t>
+  </si>
+  <si>
+    <t>As unidades de saída são padronizadas por dimensão. A coluna Unidade em 02_OUTPUTS é preenchida automaticamente pelo writer conforme basis_time_mode.</t>
+  </si>
+  <si>
+    <t>Entradas em quantidade geram saídas em kmol, kg, Nm³, MJ e kWh. Entradas em vazão geram saídas em kmol/h, kg/h, Nm³/h, MJ/h e kW. A unidade kW é usada para potência equivalente à kWh/h.</t>
+  </si>
+  <si>
+    <t>Quantidade de entrada</t>
+  </si>
+  <si>
+    <t>O significado físico de input_quantity é definido conjuntamente por input_basis_type e input_unit. O valor pode representar uma quantidade total ou uma vazão, e pode estar em base molar ou mássica.</t>
+  </si>
+  <si>
+    <t>A mesma base de entrada é aplicada globalmente a todas as linhas ativas da tabela de componentes.</t>
+  </si>
+  <si>
+    <t>input_quantity contém o valor numérico da alimentação de cada componente, interpretado segundo input_basis_type e input_unit. Para unidades com /h, input_quantity representa vazão. Para unidades sem /h, input_quantity representa quantidade total.</t>
+  </si>
+  <si>
+    <t>Use input_basis_type e input_unit de forma consistente para todos os componentes ativos. O software interpreta input_quantity como quantidade ou vazão, em base molar ou mássica, converte para kmol ou kmol/h internamente e apresenta as unidades padronizadas na aba 02_OUTPUTS.</t>
+  </si>
+  <si>
+    <t>Base de entrada</t>
   </si>
 </sst>
 </file>
@@ -1561,42 +1621,42 @@
     </row>
     <row r="6" spans="1:8" ht="43.5">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>380</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>332</v>
+        <v>379</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29.25">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="29.25">
       <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="29.25">
       <c r="A9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>12</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15">
       <c r="A10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>14</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>
@@ -1626,7 +1686,7 @@
   <sheetData>
     <row r="1" spans="1:29" ht="18">
       <c r="A1" s="26" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -1644,182 +1704,182 @@
     </row>
     <row r="3" spans="1:29" ht="15">
       <c r="A3" s="27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" s="27"/>
       <c r="C3" s="27"/>
       <c r="D3" s="27"/>
       <c r="AA3" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="AB3" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="AC3" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="45">
       <c r="A4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>21</v>
-      </c>
       <c r="AA4" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="AB4" t="s">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="AC4" t="s">
-        <v>357</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="57.75">
       <c r="A5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" t="s">
         <v>24</v>
       </c>
-      <c r="D5" t="s">
-        <v>25</v>
-      </c>
       <c r="AA5" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="AB5" t="s">
+        <v>341</v>
+      </c>
+      <c r="AC5" t="s">
         <v>348</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="43.5">
       <c r="A6" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>28</v>
-      </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="AB6" t="s">
+        <v>342</v>
+      </c>
+      <c r="AC6" t="s">
         <v>349</v>
-      </c>
-      <c r="AC6" t="s">
-        <v>356</v>
       </c>
     </row>
     <row r="7" spans="1:29" s="15" customFormat="1" ht="15">
       <c r="A7" s="35" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="B7" s="36" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="C7" s="19"/>
       <c r="AB7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AC7" t="s">
-        <v>359</v>
+        <v>352</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="129">
       <c r="A8" s="4" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>31</v>
-      </c>
       <c r="D8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AB8" s="15"/>
       <c r="AC8" s="15" t="s">
-        <v>358</v>
+        <v>351</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="72">
       <c r="A9" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" s="5">
         <v>0.95</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AC9" s="37" t="s">
-        <v>360</v>
+        <v>353</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="43.5">
       <c r="A10" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B10" s="5">
         <v>0</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="29.25">
       <c r="A11" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" s="5">
         <v>101.325</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:29" ht="43.5">
       <c r="A12" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>44</v>
-      </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" spans="1:29" ht="62.25" customHeight="1">
       <c r="A15" s="28" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="B15" s="28"/>
       <c r="C15" s="28"/>
@@ -1834,7 +1894,7 @@
     </row>
     <row r="16" spans="1:29" ht="15">
       <c r="A16" s="27" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B16" s="27"/>
       <c r="C16" s="27"/>
@@ -1852,54 +1912,54 @@
     </row>
     <row r="17" spans="1:14" ht="15">
       <c r="A17" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
+        <v>345</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>352</v>
-      </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="H17" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="I17" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="J17" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="K17" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="L17" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="L17" s="3" t="s">
+      <c r="M17" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="M17" s="3" t="s">
+      <c r="N17" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="N17" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:14" s="15" customFormat="1" ht="28.5">
       <c r="A18" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="B18" s="16" t="s">
         <v>299</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>300</v>
       </c>
       <c r="C18" s="17" t="b">
         <v>0</v>
@@ -1908,7 +1968,7 @@
         <v>0</v>
       </c>
       <c r="E18" s="16" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F18" s="16"/>
       <c r="G18" s="16"/>
@@ -1916,13 +1976,13 @@
       <c r="I18" s="16"/>
       <c r="J18" s="16"/>
       <c r="K18" s="16" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="L18" s="16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="N18" s="17" t="b">
         <v>1</v>
@@ -1930,13 +1990,13 @@
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B19" s="6" t="s">
-        <v>60</v>
-      </c>
       <c r="C19" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D19" s="6">
         <v>1</v>
@@ -1948,27 +2008,27 @@
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L19" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="M19" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="M19" s="6" t="s">
-        <v>63</v>
-      </c>
       <c r="N19" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D20" s="6">
         <v>0.5</v>
@@ -1980,27 +2040,27 @@
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L20" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="M20" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="M20" s="6" t="s">
-        <v>63</v>
-      </c>
       <c r="N20" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="21" spans="1:14">
       <c r="A21" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>66</v>
-      </c>
       <c r="C21" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D21" s="6">
         <v>0.2</v>
@@ -2012,27 +2072,27 @@
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="L21" s="6" t="s">
+      <c r="M21" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="M21" s="6" t="s">
-        <v>63</v>
-      </c>
       <c r="N21" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="28.5">
       <c r="A22" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B22" s="6" t="s">
-        <v>68</v>
-      </c>
       <c r="C22" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D22" s="6">
         <v>0.1</v>
@@ -2044,33 +2104,33 @@
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="L22" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="L22" s="6" t="s">
-        <v>62</v>
-      </c>
       <c r="M22" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>71</v>
-      </c>
       <c r="C23" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D23" s="6">
         <v>0</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
@@ -2078,27 +2138,27 @@
       <c r="I23" s="6"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="L23" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="L23" s="6" t="s">
+      <c r="M23" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="M23" s="6" t="s">
-        <v>75</v>
-      </c>
       <c r="N23" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="24" spans="1:14">
       <c r="A24" s="6" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D24" s="6">
         <v>0</v>
@@ -2120,16 +2180,16 @@
         <v>0</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="L24" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="M24" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="M24" s="6" t="s">
-        <v>75</v>
-      </c>
       <c r="N24" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25" spans="1:14">
@@ -2394,27 +2454,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1">
       <c r="A1" s="30" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
     </row>
     <row r="2" spans="1:6" ht="15">
       <c r="A2" s="29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C3" s="13" t="s">
         <v>81</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>82</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -2422,7 +2482,7 @@
     </row>
     <row r="4" spans="1:6" ht="28.5">
       <c r="A4" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" s="12" t="str">
         <f>'01_INPUTS'!B4</f>
@@ -2435,7 +2495,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B5" s="12" t="str">
         <f>'01_INPUTS'!B5</f>
@@ -2448,7 +2508,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B6" s="12" t="str">
         <f>'01_INPUTS'!B6</f>
@@ -2461,7 +2521,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B7" s="12" t="str">
         <f>'01_INPUTS'!B8</f>
@@ -2482,20 +2542,20 @@
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" s="29" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B9" s="29"/>
       <c r="C9" s="29"/>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="13" t="s">
         <v>81</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>82</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -2503,11 +2563,11 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -2515,11 +2575,11 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -2527,11 +2587,11 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2539,11 +2599,11 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="12" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -2551,18 +2611,18 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -2570,11 +2630,11 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -2590,7 +2650,7 @@
     </row>
     <row r="19" spans="1:6" ht="15">
       <c r="A19" s="31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B19" s="31"/>
       <c r="C19" s="31"/>
@@ -2600,13 +2660,13 @@
     </row>
     <row r="20" spans="1:6" ht="15">
       <c r="A20" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="C20" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -2614,7 +2674,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -2624,7 +2684,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -2634,7 +2694,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -2644,7 +2704,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
@@ -2654,15 +2714,15 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -2670,7 +2730,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
@@ -2688,7 +2748,7 @@
     </row>
     <row r="29" spans="1:6" ht="15">
       <c r="A29" s="31" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
@@ -2698,13 +2758,13 @@
     </row>
     <row r="30" spans="1:6" ht="15">
       <c r="A30" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="C30" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -2712,7 +2772,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12"/>
@@ -2722,7 +2782,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="12" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12"/>
@@ -2732,7 +2792,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -2740,12 +2800,12 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -2753,7 +2813,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="7" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -2769,7 +2829,7 @@
     </row>
     <row r="38" spans="1:6" s="7" customFormat="1" ht="15">
       <c r="A38" s="31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B38" s="31"/>
       <c r="C38" s="31"/>
@@ -2779,13 +2839,13 @@
     </row>
     <row r="39" spans="1:6" ht="15">
       <c r="A39" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="C39" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -2793,12 +2853,12 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="7" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -2806,7 +2866,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2814,7 +2874,7 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -2822,7 +2882,7 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B44" s="12"/>
       <c r="C44" s="12"/>
@@ -2832,11 +2892,11 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="12" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -2852,7 +2912,7 @@
     </row>
     <row r="47" spans="1:6" ht="15">
       <c r="A47" s="31" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B47" s="31"/>
       <c r="C47" s="31"/>
@@ -2862,13 +2922,13 @@
     </row>
     <row r="48" spans="1:6" ht="15">
       <c r="A48" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B48" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B48" s="14" t="s">
+      <c r="C48" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="C48" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
@@ -2876,7 +2936,7 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B49" s="12"/>
       <c r="C49" s="12"/>
@@ -2886,7 +2946,7 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="12"/>
@@ -2896,11 +2956,11 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
@@ -2916,7 +2976,7 @@
     </row>
     <row r="53" spans="1:6" ht="15">
       <c r="A53" s="31" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B53" s="31"/>
       <c r="C53" s="31"/>
@@ -2926,13 +2986,13 @@
     </row>
     <row r="54" spans="1:6" ht="15">
       <c r="A54" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B54" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B54" s="14" t="s">
+      <c r="C54" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -2940,7 +3000,7 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="12"/>
@@ -2950,7 +3010,7 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="12" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B56" s="12"/>
       <c r="C56" s="12"/>
@@ -2960,7 +3020,7 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="12"/>
@@ -2970,7 +3030,7 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B58" s="12"/>
       <c r="C58" s="12"/>
@@ -2980,11 +3040,11 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -2992,11 +3052,11 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B60" s="12"/>
       <c r="C60" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -3012,7 +3072,7 @@
     </row>
     <row r="62" spans="1:6" ht="15">
       <c r="A62" s="31" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B62" s="31"/>
       <c r="C62" s="31"/>
@@ -3022,13 +3082,13 @@
     </row>
     <row r="63" spans="1:6" ht="15">
       <c r="A63" s="14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B63" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="B63" s="14" t="s">
+      <c r="C63" s="14" t="s">
         <v>81</v>
-      </c>
-      <c r="C63" s="14" t="s">
-        <v>82</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
@@ -3036,11 +3096,11 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="12" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B64" s="12"/>
       <c r="C64" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
@@ -3048,11 +3108,11 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
@@ -3060,11 +3120,11 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="12" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -3072,11 +3132,11 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="12" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
@@ -3201,7 +3261,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18">
       <c r="A1" s="26" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -3216,45 +3276,45 @@
     </row>
     <row r="3" spans="1:11" ht="30">
       <c r="A3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>47</v>
-      </c>
       <c r="I3" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>136</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C4" s="2">
         <v>6</v>
@@ -3272,24 +3332,24 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>140</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>141</v>
       </c>
       <c r="C5" s="2">
         <v>12</v>
@@ -3307,24 +3367,24 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C6" s="2">
         <v>5</v>
@@ -3342,24 +3402,24 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C7" s="2">
         <v>6</v>
@@ -3377,24 +3437,24 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C8" s="2">
         <v>5</v>
@@ -3412,24 +3472,24 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C9" s="2">
         <v>6</v>
@@ -3447,24 +3507,24 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>147</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>148</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
@@ -3482,24 +3542,24 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
@@ -3517,24 +3577,24 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="2" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C12" s="2">
         <v>5</v>
@@ -3552,24 +3612,24 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>152</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>153</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
@@ -3587,24 +3647,24 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="C14" s="2">
         <v>5</v>
@@ -3622,24 +3682,24 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="C15" s="2">
         <v>3</v>
@@ -3657,24 +3717,24 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -3692,24 +3752,24 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C17" s="2">
         <v>7.3</v>
@@ -3727,24 +3787,24 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>163</v>
-      </c>
-      <c r="B18" s="2" t="s">
-        <v>164</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -3762,16 +3822,16 @@
         <v>3.5000000000000001E-3</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3797,7 +3857,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18">
       <c r="A1" s="26" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -3815,51 +3875,51 @@
     </row>
     <row r="3" spans="1:14" ht="30">
       <c r="A3" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="L3" s="3" t="s">
-        <v>178</v>
-      </c>
       <c r="M3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3873,15 +3933,15 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -3896,7 +3956,7 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -3933,7 +3993,7 @@
     </row>
     <row r="8" spans="1:14" ht="15">
       <c r="A8" s="27" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B8" s="27"/>
       <c r="C8" s="27"/>
@@ -3951,46 +4011,46 @@
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B9" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="C9" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="D9" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="E9" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="F9" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="G9" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="H9" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>189</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>190</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>191</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>192</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="M9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>194</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -7065,7 +7125,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" style="7" customWidth="1"/>
@@ -7075,7 +7135,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18">
       <c r="A1" s="26" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -7083,226 +7143,296 @@
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>197</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>198</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>199</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5">
       <c r="A4" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>318</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="D4" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="15" customFormat="1" ht="71.25">
+      <c r="A5" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="15" customFormat="1" ht="57">
+      <c r="A6" s="2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="15" customFormat="1" ht="57">
+      <c r="A7" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>373</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="15" customFormat="1" ht="57">
+      <c r="A8" s="2" t="s">
+        <v>375</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>378</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>376</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="28.5">
+      <c r="A9" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="15" customFormat="1" ht="71.25">
+      <c r="A10" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="15" customFormat="1" ht="42.75">
+      <c r="A11" s="2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>359</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="57">
+      <c r="A12" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="B12" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>329</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B14" s="22" t="s">
         <v>319</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="28.5">
-      <c r="A5" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="57">
-      <c r="A6" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="B6" s="20" t="s">
-        <v>330</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>331</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>210</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="D7" s="2" t="s">
+      <c r="C14" s="22" t="s">
+        <v>320</v>
+      </c>
+      <c r="D14" s="22" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="15" customFormat="1" ht="57">
+      <c r="A15" s="19" t="s">
+        <v>321</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>212</v>
       </c>
-    </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="22" t="s">
-        <v>320</v>
-      </c>
-      <c r="C8" s="22" t="s">
-        <v>321</v>
-      </c>
-      <c r="D8" s="22" t="s">
+      <c r="D15" s="2" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="28.5">
+      <c r="A16" s="2" t="s">
         <v>214</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" s="15" customFormat="1" ht="57">
-      <c r="A9" s="19" t="s">
+      <c r="B16" s="23" t="s">
         <v>322</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>213</v>
-      </c>
-      <c r="D9" s="2" t="s">
+      <c r="C16" s="23" t="s">
         <v>323</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="28.5">
-      <c r="A10" s="2" t="s">
+      <c r="D16" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="B10" s="23" t="s">
+    </row>
+    <row r="17" spans="1:4" s="15" customFormat="1" ht="57">
+      <c r="A17" t="s">
+        <v>327</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>324</v>
       </c>
-      <c r="C10" s="23" t="s">
+      <c r="C17" s="2" t="s">
         <v>325</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" s="15" customFormat="1" ht="57">
-      <c r="A11" t="s">
-        <v>329</v>
-      </c>
-      <c r="B11" s="2" t="s">
+      <c r="D17" s="2" t="s">
         <v>326</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>327</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="42.75">
-      <c r="A12" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>304</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>305</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="42.75">
-      <c r="A13" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>308</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>309</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="28.5">
-      <c r="A14" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>312</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>313</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="42.75">
-      <c r="A15" s="2" t="s">
-        <v>315</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>316</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>317</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="42.75">
-      <c r="A16" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>337</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="28.5">
-      <c r="A17" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>340</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>341</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="42.75">
       <c r="A18" s="2" t="s">
-        <v>343</v>
+        <v>302</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>344</v>
+        <v>303</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>345</v>
+        <v>304</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>346</v>
+        <v>305</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="42.75">
+      <c r="A19" s="2" t="s">
+        <v>306</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="28.5">
+      <c r="A20" s="2" t="s">
+        <v>310</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>311</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="42.75">
+      <c r="A21" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="42.75">
+      <c r="A22" s="2" t="s">
+        <v>332</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>334</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="42.75">
+      <c r="A23" s="2" t="s">
+        <v>336</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>337</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -7335,7 +7465,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18">
       <c r="A1" s="34" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
@@ -7372,7 +7502,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -7389,10 +7519,10 @@
     </row>
     <row r="4" spans="1:14" ht="57.75">
       <c r="A4" s="10" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -7409,10 +7539,10 @@
     </row>
     <row r="5" spans="1:14" ht="114.75">
       <c r="A5" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>220</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>221</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -7429,10 +7559,10 @@
     </row>
     <row r="6" spans="1:14" ht="29.25">
       <c r="A6" s="10" t="s">
+        <v>221</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>222</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>223</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -7465,7 +7595,7 @@
     </row>
     <row r="8" spans="1:14" ht="15">
       <c r="A8" s="33" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
@@ -7483,60 +7613,60 @@
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="D9" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="E9" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="F9" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="G9" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="H9" s="11" t="s">
         <v>230</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="I9" s="11" t="s">
         <v>231</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="J9" s="11" t="s">
         <v>232</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="K9" s="11" t="s">
         <v>233</v>
       </c>
-      <c r="K9" s="11" t="s">
+      <c r="L9" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>235</v>
       </c>
-      <c r="M9" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>236</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="85.5">
       <c r="A10" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B10" s="8" t="s">
         <v>238</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="C10" s="8" t="s">
         <v>239</v>
       </c>
-      <c r="C10" s="8" t="s">
-        <v>240</v>
-      </c>
       <c r="D10" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E10" s="8">
         <v>1</v>
@@ -7563,10 +7693,10 @@
         <v>-6.9879518072294089E-2</v>
       </c>
       <c r="M10" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="N10" s="8" t="s">
         <v>241</v>
-      </c>
-      <c r="N10" s="8" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -7587,7 +7717,7 @@
     </row>
     <row r="12" spans="1:14" ht="15">
       <c r="A12" s="33" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="33"/>
@@ -7605,60 +7735,60 @@
     </row>
     <row r="13" spans="1:14" ht="30">
       <c r="A13" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="B13" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="C13" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="C13" s="11" t="s">
-        <v>227</v>
-      </c>
       <c r="D13" s="11" t="s">
+        <v>243</v>
+      </c>
+      <c r="E13" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="F13" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="G13" s="11" t="s">
         <v>246</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="H13" s="11" t="s">
         <v>247</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="I13" s="11" t="s">
         <v>248</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="J13" s="11" t="s">
         <v>249</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="K13" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>250</v>
       </c>
-      <c r="K13" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>237</v>
-      </c>
-      <c r="M13" s="11" t="s">
+      <c r="N13" s="11" t="s">
         <v>251</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="28.5">
       <c r="A14" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="B14" s="8" t="s">
         <v>253</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="C14" s="8" t="s">
         <v>254</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="D14" s="8" t="s">
         <v>255</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>256</v>
       </c>
       <c r="E14" s="8">
         <v>490.11</v>
@@ -7679,30 +7809,30 @@
         <v>-8.4128576014130138E-2</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L14" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M14" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M14" s="8" t="s">
+      <c r="N14" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N14" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="28.5">
       <c r="A15" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>260</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="D15" s="8" t="s">
-        <v>261</v>
       </c>
       <c r="E15" s="8">
         <v>490.11</v>
@@ -7723,30 +7853,30 @@
         <v>-0.1649644901525206</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L15" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M15" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M15" s="8" t="s">
+      <c r="N15" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N15" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.5">
       <c r="A16" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>262</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>263</v>
-      </c>
       <c r="D16" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E16" s="8">
         <v>428.4</v>
@@ -7767,30 +7897,30 @@
         <v>1.6132982587243029E-2</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L16" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M16" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M16" s="8" t="s">
+      <c r="N16" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N16" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.5">
       <c r="A17" s="8" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E17" s="8">
         <v>428.4</v>
@@ -7811,30 +7941,30 @@
         <v>8.7237397338995933E-3</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L17" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M17" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M17" s="8" t="s">
+      <c r="N17" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N17" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.5">
       <c r="A18" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>265</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>266</v>
-      </c>
       <c r="D18" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E18" s="8">
         <v>484.63</v>
@@ -7855,30 +7985,30 @@
         <v>-4.5187050999701966E-3</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L18" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M18" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M18" s="8" t="s">
+      <c r="N18" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N18" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.5">
       <c r="A19" s="8" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E19" s="8">
         <v>484.63</v>
@@ -7899,30 +8029,30 @@
         <v>-4.0114456608485519E-3</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L19" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M19" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M19" s="8" t="s">
+      <c r="N19" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N19" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.5">
       <c r="A20" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>268</v>
       </c>
-      <c r="B20" s="8" t="s">
-        <v>254</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>269</v>
-      </c>
       <c r="D20" s="8" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="E20" s="8">
         <v>413.02</v>
@@ -7943,30 +8073,30 @@
         <v>-6.0227292075755966E-3</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L20" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M20" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M20" s="8" t="s">
+      <c r="N20" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N20" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.5">
       <c r="A21" s="8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="E21" s="8">
         <v>413.02</v>
@@ -7987,16 +8117,16 @@
         <v>4.72329903258944E-4</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="L21" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="M21" s="8" t="s">
         <v>257</v>
       </c>
-      <c r="M21" s="8" t="s">
+      <c r="N21" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="N21" s="8" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -8033,7 +8163,7 @@
     </row>
     <row r="24" spans="1:14" ht="15">
       <c r="A24" s="33" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B24" s="33"/>
       <c r="C24" s="33"/>
@@ -8042,19 +8172,19 @@
     </row>
     <row r="25" spans="1:14" ht="30">
       <c r="A25" s="11" t="s">
+        <v>271</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>225</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>272</v>
       </c>
-      <c r="B25" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="C25" s="11" t="s">
+      <c r="D25" s="11" t="s">
         <v>273</v>
       </c>
-      <c r="D25" s="11" t="s">
+      <c r="E25" s="11" t="s">
         <v>274</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>275</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -8068,19 +8198,19 @@
     </row>
     <row r="26" spans="1:14" ht="85.5">
       <c r="A26" s="9" t="s">
+        <v>275</v>
+      </c>
+      <c r="B26" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="C26" s="9" t="s">
         <v>277</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>278</v>
       </c>
-      <c r="D26" s="9" t="s">
+      <c r="E26" s="9" t="s">
         <v>279</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>280</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -8094,19 +8224,19 @@
     </row>
     <row r="27" spans="1:14" ht="85.5">
       <c r="A27" s="9" t="s">
+        <v>280</v>
+      </c>
+      <c r="B27" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="C27" s="9" t="s">
         <v>282</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="D27" s="9" t="s">
         <v>283</v>
       </c>
-      <c r="D27" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>284</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>285</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -8120,19 +8250,19 @@
     </row>
     <row r="28" spans="1:14" ht="71.25">
       <c r="A28" s="9" t="s">
+        <v>285</v>
+      </c>
+      <c r="B28" s="9" t="s">
         <v>286</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="C28" s="9" t="s">
         <v>287</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="D28" s="9" t="s">
         <v>288</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="E28" s="9" t="s">
         <v>289</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>290</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -8178,16 +8308,16 @@
     </row>
     <row r="31" spans="1:14" ht="15">
       <c r="A31" s="33" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="B31" s="33"/>
     </row>
     <row r="32" spans="1:14" ht="15">
       <c r="A32" s="11" t="s">
+        <v>291</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>292</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>293</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -8204,10 +8334,10 @@
     </row>
     <row r="33" spans="1:14" ht="57">
       <c r="A33" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -8224,10 +8354,10 @@
     </row>
     <row r="34" spans="1:14" ht="57">
       <c r="A34" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -8244,10 +8374,10 @@
     </row>
     <row r="35" spans="1:14" ht="42.75">
       <c r="A35" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -8264,10 +8394,10 @@
     </row>
     <row r="36" spans="1:14" ht="57">
       <c r="A36" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -8284,10 +8414,10 @@
     </row>
     <row r="37" spans="1:14" ht="57">
       <c r="A37" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>

</xml_diff>

<commit_message>
docs: polish template guidance after final review
</commit_message>
<xml_diff>
--- a/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
+++ b/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ENM\Programming\Repositories\software_BioPot-Gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D22111DD-33CE-4670-AA91-64E70B7CF2DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F9ADD9-5FF7-47AA-9FE5-15AAF138ECD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24" yWindow="-12528" windowWidth="22296" windowHeight="11904" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36" yWindow="-12540" windowWidth="22320" windowHeight="11928" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_INFORMATIVO" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="378">
   <si>
     <t>BioPot-Gas v0.6 | Informativo do template</t>
   </si>
@@ -138,15 +138,9 @@
     <t>kmol/h</t>
   </si>
   <si>
-    <t>Unidade da vazão molar usada na tabela. Use kmol ou kmol/h para obter kg e Nm³ diretamente.</t>
-  </si>
-  <si>
     <t>carbon_conversion</t>
   </si>
   <si>
-    <t>Fração do carbono direcionada à formação de biogás</t>
-  </si>
-  <si>
     <t>TRUE</t>
   </si>
   <si>
@@ -169,15 +163,6 @@
   </si>
   <si>
     <t>kWh_per_MJ</t>
-  </si>
-  <si>
-    <t>report_units</t>
-  </si>
-  <si>
-    <t>Nm3, MJ, kWh</t>
-  </si>
-  <si>
-    <t>Unidades principais do relatório</t>
   </si>
   <si>
     <t>Tabela de componentes, substratos e água disponível</t>
@@ -1192,6 +1177,12 @@
   </si>
   <si>
     <t>Base de entrada</t>
+  </si>
+  <si>
+    <t>Base da unidade de entrada. Bases aceitas são mássicas ou molares.</t>
+  </si>
+  <si>
+    <t>Unidade de entrada do input para o cálculo. São aceitos quantidades totais ou taxas (vazão).</t>
   </si>
 </sst>
 </file>
@@ -1621,10 +1612,10 @@
     </row>
     <row r="6" spans="1:8" ht="43.5">
       <c r="A6" s="1" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29.25">
@@ -1669,7 +1660,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AC38"/>
+  <dimension ref="A1:AC37"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="22" style="7" customWidth="1"/>
@@ -1682,6 +1673,7 @@
     <col min="12" max="12" width="20" style="7" customWidth="1"/>
     <col min="13" max="13" width="32" style="7" customWidth="1"/>
     <col min="14" max="14" width="12" style="7" customWidth="1"/>
+    <col min="27" max="29" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
@@ -1710,13 +1702,13 @@
       <c r="C3" s="27"/>
       <c r="D3" s="27"/>
       <c r="AA3" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="AB3" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="AC3" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="45">
@@ -1733,13 +1725,13 @@
         <v>20</v>
       </c>
       <c r="AA4" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="AB4" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="AC4" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="57.75">
@@ -1756,13 +1748,13 @@
         <v>24</v>
       </c>
       <c r="AA5" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="AB5" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="AC5" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="43.5">
@@ -1779,71 +1771,76 @@
         <v>24</v>
       </c>
       <c r="AB6" t="s">
+        <v>337</v>
+      </c>
+      <c r="AC6" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="7" spans="1:29" s="15" customFormat="1" ht="100.5">
+      <c r="A7" s="35" t="s">
+        <v>338</v>
+      </c>
+      <c r="B7" s="36" t="s">
         <v>342</v>
       </c>
-      <c r="AC6" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="7" spans="1:29" s="15" customFormat="1" ht="15">
-      <c r="A7" s="35" t="s">
-        <v>343</v>
-      </c>
-      <c r="B7" s="36" t="s">
-        <v>347</v>
-      </c>
-      <c r="C7" s="19"/>
+      <c r="C7" s="19" t="s">
+        <v>376</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>20</v>
+      </c>
       <c r="AB7" t="s">
         <v>29</v>
       </c>
       <c r="AC7" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="129">
       <c r="A8" s="4" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>30</v>
+        <v>377</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
       </c>
       <c r="AB8" s="15"/>
       <c r="AC8" s="15" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="72">
       <c r="A9" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B9" s="5">
         <v>0.95</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>32</v>
+        <v>199</v>
       </c>
       <c r="D9" t="s">
         <v>20</v>
       </c>
       <c r="AC9" s="37" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="43.5">
       <c r="A10" s="4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B10" s="5">
         <v>0</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D10" t="s">
         <v>20</v>
@@ -1851,141 +1848,159 @@
     </row>
     <row r="11" spans="1:29" ht="29.25">
       <c r="A11" s="4" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B11" s="5">
         <v>101.325</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D11" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:29" ht="43.5">
-      <c r="A12" s="4" t="s">
+    <row r="14" spans="1:29" ht="62.25" customHeight="1">
+      <c r="A14" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="B14" s="28"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
+      <c r="E14" s="28"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="28"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="28"/>
+      <c r="K14" s="28"/>
+    </row>
+    <row r="15" spans="1:29" ht="15">
+      <c r="A15" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="27"/>
+      <c r="C15" s="27"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="27"/>
+      <c r="F15" s="27"/>
+      <c r="G15" s="27"/>
+      <c r="H15" s="27"/>
+      <c r="I15" s="27"/>
+      <c r="J15" s="27"/>
+      <c r="K15" s="27"/>
+      <c r="L15" s="27"/>
+      <c r="M15" s="27"/>
+      <c r="N15" s="27"/>
+    </row>
+    <row r="16" spans="1:29" ht="15">
+      <c r="A16" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="D16" s="3" t="s">
+        <v>340</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="15" spans="1:29" ht="62.25" customHeight="1">
-      <c r="A15" s="28" t="s">
-        <v>331</v>
-      </c>
-      <c r="B15" s="28"/>
-      <c r="C15" s="28"/>
-      <c r="D15" s="28"/>
-      <c r="E15" s="28"/>
-      <c r="F15" s="28"/>
-      <c r="G15" s="28"/>
-      <c r="H15" s="28"/>
-      <c r="I15" s="28"/>
-      <c r="J15" s="28"/>
-      <c r="K15" s="28"/>
-    </row>
-    <row r="16" spans="1:29" ht="15">
-      <c r="A16" s="27" t="s">
+      <c r="F16" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="27"/>
-      <c r="C16" s="27"/>
-      <c r="D16" s="27"/>
-      <c r="E16" s="27"/>
-      <c r="F16" s="27"/>
-      <c r="G16" s="27"/>
-      <c r="H16" s="27"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="27"/>
-      <c r="K16" s="27"/>
-      <c r="L16" s="27"/>
-      <c r="M16" s="27"/>
-      <c r="N16" s="27"/>
-    </row>
-    <row r="17" spans="1:14" ht="15">
-      <c r="A17" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="I16" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>345</v>
-      </c>
-      <c r="E17" s="3" t="s">
+      <c r="J16" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="J17" s="3" t="s">
+    </row>
+    <row r="17" spans="1:14" s="15" customFormat="1" ht="28.5">
+      <c r="A17" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>294</v>
+      </c>
+      <c r="C17" s="17" t="b">
+        <v>0</v>
+      </c>
+      <c r="D17" s="16">
+        <v>0</v>
+      </c>
+      <c r="E17" s="16" t="s">
+        <v>295</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16"/>
+      <c r="H17" s="16"/>
+      <c r="I17" s="16"/>
+      <c r="J17" s="16"/>
+      <c r="K17" s="16" t="s">
+        <v>293</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>296</v>
+      </c>
+      <c r="N17" s="17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14">
+      <c r="A18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="B18" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="L17" s="3" t="s">
+      <c r="C18" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="6">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+      <c r="K18" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="M17" s="3" t="s">
+      <c r="L18" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="N17" s="3" t="s">
+      <c r="M18" s="6" t="s">
         <v>57</v>
       </c>
-    </row>
-    <row r="18" spans="1:14" s="15" customFormat="1" ht="28.5">
-      <c r="A18" s="16" t="s">
-        <v>298</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>299</v>
-      </c>
-      <c r="C18" s="17" t="b">
-        <v>0</v>
-      </c>
-      <c r="D18" s="16">
-        <v>0</v>
-      </c>
-      <c r="E18" s="16" t="s">
-        <v>300</v>
-      </c>
-      <c r="F18" s="16"/>
-      <c r="G18" s="16"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16" t="s">
-        <v>298</v>
-      </c>
-      <c r="L18" s="16" t="s">
-        <v>73</v>
-      </c>
-      <c r="M18" s="16" t="s">
-        <v>301</v>
-      </c>
-      <c r="N18" s="17" t="b">
-        <v>1</v>
+      <c r="N18" s="6" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="19" spans="1:14">
@@ -1993,13 +2008,13 @@
         <v>58</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D19" s="6">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
@@ -2008,30 +2023,30 @@
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="L19" s="6" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="M19" s="6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="N19" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D20" s="6">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="6"/>
@@ -2040,30 +2055,30 @@
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="L20" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="M20" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="N20" s="6" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" ht="28.5">
+      <c r="A21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="M20" s="6" t="s">
+      <c r="B21" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="N20" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14">
-      <c r="A21" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>65</v>
-      </c>
       <c r="C21" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D21" s="6">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
@@ -2072,125 +2087,109 @@
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="L21" s="6" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="M21" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="28.5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14">
       <c r="A22" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D22" s="6">
+        <v>0</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="B22" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="E22" s="6"/>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
       <c r="H22" s="6"/>
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="L22" s="6" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="M22" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D23" s="6">
         <v>0</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="6"/>
+      <c r="F23" s="6">
+        <v>6</v>
+      </c>
+      <c r="G23" s="6">
+        <v>10</v>
+      </c>
+      <c r="H23" s="6">
+        <v>5</v>
+      </c>
+      <c r="I23" s="6">
+        <v>0</v>
+      </c>
+      <c r="J23" s="6">
+        <v>0</v>
+      </c>
+      <c r="K23" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="F23" s="6"/>
-      <c r="G23" s="6"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
-      <c r="K23" s="6" t="s">
-        <v>72</v>
-      </c>
       <c r="L23" s="6" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="M23" s="6" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N23" s="6" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="24" spans="1:14">
-      <c r="A24" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="6">
-        <v>0</v>
-      </c>
-      <c r="E24" s="6"/>
-      <c r="F24" s="6">
-        <v>6</v>
-      </c>
-      <c r="G24" s="6">
-        <v>10</v>
-      </c>
-      <c r="H24" s="6">
-        <v>5</v>
-      </c>
-      <c r="I24" s="6">
-        <v>0</v>
-      </c>
-      <c r="J24" s="6">
-        <v>0</v>
-      </c>
-      <c r="K24" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="L24" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="M24" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="N24" s="6" t="s">
-        <v>34</v>
-      </c>
+      <c r="A24" s="18"/>
+      <c r="B24" s="18"/>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18"/>
+      <c r="E24" s="18"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18"/>
+      <c r="L24" s="18"/>
+      <c r="M24" s="18"/>
+      <c r="N24" s="18"/>
     </row>
     <row r="25" spans="1:14">
       <c r="A25" s="18"/>
@@ -2400,34 +2399,18 @@
       <c r="M37" s="18"/>
       <c r="N37" s="18"/>
     </row>
-    <row r="38" spans="1:14">
-      <c r="A38" s="18"/>
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
-      <c r="I38" s="18"/>
-      <c r="J38" s="18"/>
-      <c r="K38" s="18"/>
-      <c r="L38" s="18"/>
-      <c r="M38" s="18"/>
-      <c r="N38" s="18"/>
-    </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A16:N16"/>
+    <mergeCell ref="A15:N15"/>
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A15:K15"/>
+    <mergeCell ref="A14:K14"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation type="list" sqref="C19:C198 N19:N198" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" sqref="C18:C197 N18:N197" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation type="list" sqref="K19:K198" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" sqref="K18:K197" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>"DATABASE,FORMULA,ELEMENTS"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B8" xr:uid="{A6C2391F-5F62-4932-8555-2C756A0F9999}">
@@ -2454,27 +2437,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1">
       <c r="A1" s="30" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B1" s="30"/>
       <c r="C1" s="30"/>
     </row>
     <row r="2" spans="1:6" ht="15">
       <c r="A2" s="29" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="13" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B3" s="13" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -2542,20 +2525,20 @@
     </row>
     <row r="9" spans="1:6" ht="15">
       <c r="A9" s="29" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B9" s="29"/>
       <c r="C9" s="29"/>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="13" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -2563,11 +2546,11 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -2575,11 +2558,11 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="12" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -2587,11 +2570,11 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="12" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2599,11 +2582,11 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="12" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -2611,18 +2594,18 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -2630,11 +2613,11 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="12" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -2650,7 +2633,7 @@
     </row>
     <row r="19" spans="1:6" ht="15">
       <c r="A19" s="31" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B19" s="31"/>
       <c r="C19" s="31"/>
@@ -2660,13 +2643,13 @@
     </row>
     <row r="20" spans="1:6" ht="15">
       <c r="A20" s="14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -2674,7 +2657,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="12" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -2684,7 +2667,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="12" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -2694,7 +2677,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="12" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -2704,7 +2687,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="12" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
@@ -2714,15 +2697,15 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="7" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="7" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -2730,7 +2713,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="12" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
@@ -2748,7 +2731,7 @@
     </row>
     <row r="29" spans="1:6" ht="15">
       <c r="A29" s="31" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B29" s="31"/>
       <c r="C29" s="31"/>
@@ -2758,13 +2741,13 @@
     </row>
     <row r="30" spans="1:6" ht="15">
       <c r="A30" s="14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -2772,7 +2755,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="12" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12"/>
@@ -2782,7 +2765,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="12" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12"/>
@@ -2792,7 +2775,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="7" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -2800,12 +2783,12 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="7" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="7" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -2813,7 +2796,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="7" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -2829,7 +2812,7 @@
     </row>
     <row r="38" spans="1:6" s="7" customFormat="1" ht="15">
       <c r="A38" s="31" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B38" s="31"/>
       <c r="C38" s="31"/>
@@ -2839,13 +2822,13 @@
     </row>
     <row r="39" spans="1:6" ht="15">
       <c r="A39" s="14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -2853,12 +2836,12 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="7" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="7" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -2866,7 +2849,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="7" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2874,7 +2857,7 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="7" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -2882,7 +2865,7 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="12" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B44" s="12"/>
       <c r="C44" s="12"/>
@@ -2892,11 +2875,11 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="12" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="12" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -2912,7 +2895,7 @@
     </row>
     <row r="47" spans="1:6" ht="15">
       <c r="A47" s="31" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B47" s="31"/>
       <c r="C47" s="31"/>
@@ -2922,13 +2905,13 @@
     </row>
     <row r="48" spans="1:6" ht="15">
       <c r="A48" s="14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B48" s="14" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C48" s="14" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
@@ -2936,7 +2919,7 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="12" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B49" s="12"/>
       <c r="C49" s="12"/>
@@ -2946,7 +2929,7 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="12" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="12"/>
@@ -2956,11 +2939,11 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="12" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="12" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
@@ -2976,7 +2959,7 @@
     </row>
     <row r="53" spans="1:6" ht="15">
       <c r="A53" s="31" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B53" s="31"/>
       <c r="C53" s="31"/>
@@ -2986,13 +2969,13 @@
     </row>
     <row r="54" spans="1:6" ht="15">
       <c r="A54" s="14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B54" s="14" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C54" s="14" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -3000,7 +2983,7 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="12" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="12"/>
@@ -3010,7 +2993,7 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="12" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B56" s="12"/>
       <c r="C56" s="12"/>
@@ -3020,7 +3003,7 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="12" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="12"/>
@@ -3030,7 +3013,7 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="12" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B58" s="12"/>
       <c r="C58" s="12"/>
@@ -3040,11 +3023,11 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="12" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -3052,11 +3035,11 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="12" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B60" s="12"/>
       <c r="C60" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -3072,7 +3055,7 @@
     </row>
     <row r="62" spans="1:6" ht="15">
       <c r="A62" s="31" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B62" s="31"/>
       <c r="C62" s="31"/>
@@ -3082,13 +3065,13 @@
     </row>
     <row r="63" spans="1:6" ht="15">
       <c r="A63" s="14" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B63" s="14" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C63" s="14" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
@@ -3096,11 +3079,11 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="12" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B64" s="12"/>
       <c r="C64" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
@@ -3108,11 +3091,11 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="12" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
@@ -3120,11 +3103,11 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="12" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -3132,11 +3115,11 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="12" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="12" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
@@ -3261,7 +3244,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="18">
       <c r="A1" s="26" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B1" s="32"/>
       <c r="C1" s="32"/>
@@ -3276,45 +3259,45 @@
     </row>
     <row r="3" spans="1:11" ht="30">
       <c r="A3" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="E3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>53</v>
-      </c>
       <c r="H3" s="3" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C4" s="2">
         <v>6</v>
@@ -3332,24 +3315,24 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C5" s="2">
         <v>12</v>
@@ -3367,24 +3350,24 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C6" s="2">
         <v>5</v>
@@ -3402,24 +3385,24 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C7" s="2">
         <v>6</v>
@@ -3437,24 +3420,24 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C8" s="2">
         <v>5</v>
@@ -3472,24 +3455,24 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="2" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C9" s="2">
         <v>6</v>
@@ -3507,24 +3490,24 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="2" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
@@ -3542,24 +3525,24 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
@@ -3577,24 +3560,24 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="2" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C12" s="2">
         <v>5</v>
@@ -3612,24 +3595,24 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="2" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
@@ -3647,24 +3630,24 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="2" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C14" s="2">
         <v>5</v>
@@ -3682,24 +3665,24 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="C15" s="2">
         <v>3</v>
@@ -3717,24 +3700,24 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="2" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -3752,24 +3735,24 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="2" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="C17" s="2">
         <v>7.3</v>
@@ -3787,24 +3770,24 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="2" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -3822,16 +3805,16 @@
         <v>3.5000000000000001E-3</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -3857,7 +3840,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18">
       <c r="A1" s="26" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -3875,51 +3858,51 @@
     </row>
     <row r="3" spans="1:14" ht="30">
       <c r="A3" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>177</v>
-      </c>
       <c r="M3" s="3" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3933,15 +3916,15 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -3956,7 +3939,7 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -3993,7 +3976,7 @@
     </row>
     <row r="8" spans="1:14" ht="15">
       <c r="A8" s="27" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="B8" s="27"/>
       <c r="C8" s="27"/>
@@ -4011,46 +3994,46 @@
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="13" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="B9" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="G9" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="H9" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>187</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>188</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>189</v>
-      </c>
-      <c r="J9" s="13" t="s">
-        <v>190</v>
-      </c>
-      <c r="K9" s="13" t="s">
-        <v>191</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>192</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>193</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -7135,7 +7118,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="18">
       <c r="A1" s="26" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="B1" s="26"/>
       <c r="C1" s="26"/>
@@ -7143,142 +7126,142 @@
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="3" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="15" customFormat="1" ht="71.25">
       <c r="A5" s="2" t="s">
-        <v>363</v>
+        <v>358</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>364</v>
+        <v>359</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A6" s="2" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A7" s="2" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>373</v>
+        <v>368</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>372</v>
+        <v>367</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A8" s="2" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28.5">
       <c r="A9" s="2" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="15" customFormat="1" ht="71.25">
       <c r="A10" s="2" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="15" customFormat="1" ht="42.75">
       <c r="A11" s="2" t="s">
-        <v>358</v>
+        <v>353</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>359</v>
+        <v>354</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="57">
       <c r="A12" s="2" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>329</v>
+        <v>324</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -7286,13 +7269,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -7300,139 +7283,139 @@
         <v>11</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>319</v>
+        <v>314</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="15" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A15" s="19" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="28.5">
       <c r="A16" s="2" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>323</v>
+        <v>318</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="17" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A17" t="s">
-        <v>327</v>
+        <v>322</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>325</v>
+        <v>320</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="42.75">
       <c r="A18" s="2" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="42.75">
       <c r="A19" s="2" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="28.5">
       <c r="A20" s="2" t="s">
-        <v>310</v>
+        <v>305</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>311</v>
+        <v>306</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>313</v>
+        <v>308</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="42.75">
       <c r="A21" s="2" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>317</v>
+        <v>312</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="42.75">
       <c r="A22" s="2" t="s">
-        <v>332</v>
+        <v>327</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="42.75">
       <c r="A23" s="2" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -7465,7 +7448,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="18">
       <c r="A1" s="34" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B1" s="34"/>
       <c r="C1" s="34"/>
@@ -7502,7 +7485,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -7519,10 +7502,10 @@
     </row>
     <row r="4" spans="1:14" ht="57.75">
       <c r="A4" s="10" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -7539,10 +7522,10 @@
     </row>
     <row r="5" spans="1:14" ht="114.75">
       <c r="A5" s="10" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -7559,10 +7542,10 @@
     </row>
     <row r="6" spans="1:14" ht="29.25">
       <c r="A6" s="10" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -7595,7 +7578,7 @@
     </row>
     <row r="8" spans="1:14" ht="15">
       <c r="A8" s="33" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
@@ -7613,60 +7596,60 @@
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="11" t="s">
+        <v>219</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>220</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="D9" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>223</v>
+      </c>
+      <c r="G9" s="11" t="s">
         <v>224</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="H9" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="I9" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="J9" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="K9" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="L9" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>230</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>231</v>
-      </c>
-      <c r="J9" s="11" t="s">
-        <v>232</v>
-      </c>
-      <c r="K9" s="11" t="s">
-        <v>233</v>
-      </c>
-      <c r="L9" s="11" t="s">
-        <v>234</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="85.5">
       <c r="A10" s="8" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="E10" s="8">
         <v>1</v>
@@ -7693,10 +7676,10 @@
         <v>-6.9879518072294089E-2</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -7717,7 +7700,7 @@
     </row>
     <row r="12" spans="1:14" ht="15">
       <c r="A12" s="33" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="B12" s="33"/>
       <c r="C12" s="33"/>
@@ -7735,60 +7718,60 @@
     </row>
     <row r="13" spans="1:14" ht="30">
       <c r="A13" s="11" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="D13" s="11" t="s">
+        <v>238</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>239</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>241</v>
+      </c>
+      <c r="H13" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="I13" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="J13" s="11" t="s">
         <v>244</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="K13" s="11" t="s">
+        <v>230</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>245</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="N13" s="11" t="s">
         <v>246</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>247</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="J13" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>235</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>250</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="28.5">
       <c r="A14" s="8" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E14" s="8">
         <v>490.11</v>
@@ -7809,30 +7792,30 @@
         <v>-8.4128576014130138E-2</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L14" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M14" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N14" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="28.5">
       <c r="A15" s="8" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E15" s="8">
         <v>490.11</v>
@@ -7853,30 +7836,30 @@
         <v>-0.1649644901525206</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M15" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N15" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.5">
       <c r="A16" s="8" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E16" s="8">
         <v>428.4</v>
@@ -7897,30 +7880,30 @@
         <v>1.6132982587243029E-2</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M16" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N16" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.5">
       <c r="A17" s="8" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E17" s="8">
         <v>428.4</v>
@@ -7941,30 +7924,30 @@
         <v>8.7237397338995933E-3</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L17" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M17" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N17" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.5">
       <c r="A18" s="8" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D18" s="8" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E18" s="8">
         <v>484.63</v>
@@ -7985,30 +7968,30 @@
         <v>-4.5187050999701966E-3</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L18" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M18" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N18" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.5">
       <c r="A19" s="8" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E19" s="8">
         <v>484.63</v>
@@ -8029,30 +8012,30 @@
         <v>-4.0114456608485519E-3</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L19" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M19" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N19" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.5">
       <c r="A20" s="8" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D20" s="8" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="E20" s="8">
         <v>413.02</v>
@@ -8073,30 +8056,30 @@
         <v>-6.0227292075755966E-3</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M20" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N20" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.5">
       <c r="A21" s="8" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="E21" s="8">
         <v>413.02</v>
@@ -8117,16 +8100,16 @@
         <v>4.72329903258944E-4</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M21" s="8" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="N21" s="8" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -8163,7 +8146,7 @@
     </row>
     <row r="24" spans="1:14" ht="15">
       <c r="A24" s="33" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
       <c r="B24" s="33"/>
       <c r="C24" s="33"/>
@@ -8172,19 +8155,19 @@
     </row>
     <row r="25" spans="1:14" ht="30">
       <c r="A25" s="11" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
       <c r="D25" s="11" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="E25" s="11" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -8198,19 +8181,19 @@
     </row>
     <row r="26" spans="1:14" ht="85.5">
       <c r="A26" s="9" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -8224,19 +8207,19 @@
     </row>
     <row r="27" spans="1:14" ht="85.5">
       <c r="A27" s="9" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -8250,19 +8233,19 @@
     </row>
     <row r="28" spans="1:14" ht="71.25">
       <c r="A28" s="9" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="E28" s="9" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -8308,16 +8291,16 @@
     </row>
     <row r="31" spans="1:14" ht="15">
       <c r="A31" s="33" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="B31" s="33"/>
     </row>
     <row r="32" spans="1:14" ht="15">
       <c r="A32" s="11" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -8334,10 +8317,10 @@
     </row>
     <row r="33" spans="1:14" ht="57">
       <c r="A33" s="2" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -8354,10 +8337,10 @@
     </row>
     <row r="34" spans="1:14" ht="57">
       <c r="A34" s="2" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -8374,10 +8357,10 @@
     </row>
     <row r="35" spans="1:14" ht="42.75">
       <c r="A35" s="2" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -8394,10 +8377,10 @@
     </row>
     <row r="36" spans="1:14" ht="57">
       <c r="A36" s="2" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -8414,10 +8397,10 @@
     </row>
     <row r="37" spans="1:14" ht="57">
       <c r="A37" s="2" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>

</xml_diff>

<commit_message>
docs: update release notes for v0.6.1
</commit_message>
<xml_diff>
--- a/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
+++ b/BioPot-Gas_Input_Template_v6_validation_benchmarks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ENM\Programming\Repositories\software_BioPot-Gas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6F9ADD9-5FF7-47AA-9FE5-15AAF138ECD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B98113AA-7F3F-4ADF-8987-EA532285BE09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36" yWindow="-12540" windowWidth="22320" windowHeight="11928" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_INFORMATIVO" sheetId="1" r:id="rId1"/>
@@ -102,9 +102,6 @@
     <t>Project_name</t>
   </si>
   <si>
-    <t>Example BioPot-Gas v0.5</t>
-  </si>
-  <si>
     <t>Nome do estudo ou cenário</t>
   </si>
   <si>
@@ -430,9 +427,6 @@
   </si>
   <si>
     <t>carbon_conversion_note</t>
-  </si>
-  <si>
-    <t>BioPot-Gas v0.5 | Banco de Componentes</t>
   </si>
   <si>
     <t>default_degradable</t>
@@ -1183,6 +1177,12 @@
   </si>
   <si>
     <t>Unidade de entrada do input para o cálculo. São aceitos quantidades totais ou taxas (vazão).</t>
+  </si>
+  <si>
+    <t>BioPot-Gas v0.6 | Banco de Componentes</t>
+  </si>
+  <si>
+    <t>Example BioPot-Gas v0.6</t>
   </si>
 </sst>
 </file>
@@ -1372,6 +1372,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1397,9 +1400,6 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1575,16 +1575,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="18">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
     </row>
     <row r="3" spans="1:8" ht="29.25">
       <c r="A3" s="1" t="s">
@@ -1612,10 +1612,10 @@
     </row>
     <row r="6" spans="1:8" ht="43.5">
       <c r="A6" s="1" t="s">
-        <v>375</v>
+        <v>373</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="29.25">
@@ -1677,38 +1677,38 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:29" ht="18">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
     </row>
     <row r="3" spans="1:29" ht="15">
-      <c r="A3" s="27" t="s">
+      <c r="A3" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
+      <c r="B3" s="30"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
       <c r="AA3" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="AB3" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AC3" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
     </row>
     <row r="4" spans="1:29" ht="45">
@@ -1716,233 +1716,233 @@
         <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="AA4" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="AB4" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="AC4" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
     <row r="5" spans="1:29" ht="57.75">
       <c r="A5" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="D5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" t="s">
-        <v>24</v>
-      </c>
       <c r="AA5" t="s">
+        <v>339</v>
+      </c>
+      <c r="AB5" t="s">
+        <v>334</v>
+      </c>
+      <c r="AC5" t="s">
         <v>341</v>
-      </c>
-      <c r="AB5" t="s">
-        <v>336</v>
-      </c>
-      <c r="AC5" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="6" spans="1:29" ht="43.5">
       <c r="A6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AB6" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="AC6" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
     </row>
     <row r="7" spans="1:29" s="15" customFormat="1" ht="100.5">
-      <c r="A7" s="35" t="s">
-        <v>338</v>
-      </c>
-      <c r="B7" s="36" t="s">
-        <v>342</v>
+      <c r="A7" s="26" t="s">
+        <v>336</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>340</v>
       </c>
       <c r="C7" s="19" t="s">
-        <v>376</v>
+        <v>374</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AB7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="AC7" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
     </row>
     <row r="8" spans="1:29" ht="129">
       <c r="A8" s="4" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>377</v>
+        <v>375</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AB8" s="15"/>
       <c r="AC8" s="15" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
     </row>
     <row r="9" spans="1:29" ht="72">
       <c r="A9" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="5">
         <v>0.95</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
-      </c>
-      <c r="AC9" s="37" t="s">
-        <v>348</v>
+        <v>19</v>
+      </c>
+      <c r="AC9" s="28" t="s">
+        <v>346</v>
       </c>
     </row>
     <row r="10" spans="1:29" ht="43.5">
       <c r="A10" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="5">
         <v>0</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:29" ht="29.25">
       <c r="A11" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B11" s="5">
         <v>101.325</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:29" ht="62.25" customHeight="1">
-      <c r="A14" s="28" t="s">
-        <v>326</v>
-      </c>
-      <c r="B14" s="28"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="28"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="28"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="28"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="28"/>
-      <c r="K14" s="28"/>
+      <c r="A14" s="31" t="s">
+        <v>324</v>
+      </c>
+      <c r="B14" s="31"/>
+      <c r="C14" s="31"/>
+      <c r="D14" s="31"/>
+      <c r="E14" s="31"/>
+      <c r="F14" s="31"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+      <c r="I14" s="31"/>
+      <c r="J14" s="31"/>
+      <c r="K14" s="31"/>
     </row>
     <row r="15" spans="1:29" ht="15">
-      <c r="A15" s="27" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="27"/>
-      <c r="C15" s="27"/>
-      <c r="D15" s="27"/>
-      <c r="E15" s="27"/>
-      <c r="F15" s="27"/>
-      <c r="G15" s="27"/>
-      <c r="H15" s="27"/>
-      <c r="I15" s="27"/>
-      <c r="J15" s="27"/>
-      <c r="K15" s="27"/>
-      <c r="L15" s="27"/>
-      <c r="M15" s="27"/>
-      <c r="N15" s="27"/>
+      <c r="A15" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="B15" s="30"/>
+      <c r="C15" s="30"/>
+      <c r="D15" s="30"/>
+      <c r="E15" s="30"/>
+      <c r="F15" s="30"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="30"/>
+      <c r="N15" s="30"/>
     </row>
     <row r="16" spans="1:29" ht="15">
       <c r="A16" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
+        <v>338</v>
+      </c>
+      <c r="E16" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="D16" s="3" t="s">
-        <v>340</v>
-      </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="I16" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="I16" s="3" t="s">
+      <c r="J16" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:14" s="15" customFormat="1" ht="28.5">
       <c r="A17" s="16" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C17" s="17" t="b">
         <v>0</v>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
       <c r="E17" s="16" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="F17" s="16"/>
       <c r="G17" s="16"/>
@@ -1959,13 +1959,13 @@
       <c r="I17" s="16"/>
       <c r="J17" s="16"/>
       <c r="K17" s="16" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="L17" s="16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="N17" s="17" t="b">
         <v>1</v>
@@ -1973,13 +1973,13 @@
     </row>
     <row r="18" spans="1:14">
       <c r="A18" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>54</v>
-      </c>
       <c r="C18" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D18" s="6">
         <v>1</v>
@@ -1991,27 +1991,27 @@
       <c r="I18" s="6"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L18" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="L18" s="6" t="s">
+      <c r="M18" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="M18" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="N18" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19" spans="1:14">
       <c r="A19" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D19" s="6">
         <v>0.5</v>
@@ -2023,27 +2023,27 @@
       <c r="I19" s="6"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L19" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="L19" s="6" t="s">
+      <c r="M19" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="M19" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="N19" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="20" spans="1:14">
       <c r="A20" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B20" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="B20" s="6" t="s">
-        <v>60</v>
-      </c>
       <c r="C20" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D20" s="6">
         <v>0.2</v>
@@ -2055,27 +2055,27 @@
       <c r="I20" s="6"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L20" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="L20" s="6" t="s">
+      <c r="M20" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="M20" s="6" t="s">
-        <v>57</v>
-      </c>
       <c r="N20" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.5">
       <c r="A21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>62</v>
-      </c>
       <c r="C21" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D21" s="6">
         <v>0.1</v>
@@ -2087,33 +2087,33 @@
       <c r="I21" s="6"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="L21" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="L21" s="6" t="s">
-        <v>56</v>
-      </c>
       <c r="M21" s="6" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="N21" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="22" spans="1:14">
       <c r="A22" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B22" s="6" t="s">
-        <v>65</v>
-      </c>
       <c r="C22" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D22" s="6">
         <v>0</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6"/>
@@ -2121,27 +2121,27 @@
       <c r="I22" s="6"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="L22" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="L22" s="6" t="s">
+      <c r="M22" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M22" s="6" t="s">
-        <v>69</v>
-      </c>
       <c r="N22" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="23" spans="1:14">
       <c r="A23" s="6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D23" s="6">
         <v>0</v>
@@ -2163,16 +2163,16 @@
         <v>0</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="L23" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="M23" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="M23" s="6" t="s">
-        <v>69</v>
-      </c>
       <c r="N23" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="24" spans="1:14">
@@ -2436,28 +2436,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="36" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="33" t="s">
+        <v>71</v>
+      </c>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+    </row>
+    <row r="2" spans="1:6" ht="15">
+      <c r="A2" s="32" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
-    </row>
-    <row r="2" spans="1:6" ht="15">
-      <c r="A2" s="29" t="s">
-        <v>73</v>
-      </c>
-      <c r="B2" s="29"/>
-      <c r="C2" s="29"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
     </row>
     <row r="3" spans="1:6" ht="15">
       <c r="A3" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="13" t="s">
+      <c r="C3" s="13" t="s">
         <v>75</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>76</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="B4" s="12" t="str">
         <f>'01_INPUTS'!B4</f>
-        <v>Example BioPot-Gas v0.5</v>
+        <v>Example BioPot-Gas v0.6</v>
       </c>
       <c r="C4" s="12"/>
       <c r="D4" s="2"/>
@@ -2478,7 +2478,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" s="12" t="str">
         <f>'01_INPUTS'!B5</f>
@@ -2491,7 +2491,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B6" s="12" t="str">
         <f>'01_INPUTS'!B6</f>
@@ -2504,7 +2504,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B7" s="12" t="str">
         <f>'01_INPUTS'!B8</f>
@@ -2524,21 +2524,21 @@
       <c r="F8" s="2"/>
     </row>
     <row r="9" spans="1:6" ht="15">
-      <c r="A9" s="29" t="s">
-        <v>77</v>
-      </c>
-      <c r="B9" s="29"/>
-      <c r="C9" s="29"/>
+      <c r="A9" s="32" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
     </row>
     <row r="10" spans="1:6" ht="15">
       <c r="A10" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="C10" s="13" t="s">
         <v>75</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>76</v>
       </c>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
@@ -2546,11 +2546,11 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
@@ -2558,11 +2558,11 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -2570,11 +2570,11 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -2582,11 +2582,11 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -2594,18 +2594,18 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
@@ -2613,11 +2613,11 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B17" s="12"/>
       <c r="C17" s="12" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
@@ -2632,24 +2632,24 @@
       <c r="F18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="15">
-      <c r="A19" s="31" t="s">
-        <v>87</v>
-      </c>
-      <c r="B19" s="31"/>
-      <c r="C19" s="31"/>
+      <c r="A19" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="B19" s="34"/>
+      <c r="C19" s="34"/>
       <c r="D19" s="2"/>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
     <row r="20" spans="1:6" ht="15">
       <c r="A20" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B20" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B20" s="14" t="s">
+      <c r="C20" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -2657,7 +2657,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="12" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -2667,7 +2667,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="12" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -2677,7 +2677,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B23" s="12"/>
       <c r="C23" s="12"/>
@@ -2687,7 +2687,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="12" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B24" s="12"/>
       <c r="C24" s="12"/>
@@ -2697,15 +2697,15 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="7" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -2713,7 +2713,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B27" s="12"/>
       <c r="C27" s="12"/>
@@ -2730,24 +2730,24 @@
       <c r="F28" s="2"/>
     </row>
     <row r="29" spans="1:6" ht="15">
-      <c r="A29" s="31" t="s">
-        <v>95</v>
-      </c>
-      <c r="B29" s="31"/>
-      <c r="C29" s="31"/>
+      <c r="A29" s="34" t="s">
+        <v>94</v>
+      </c>
+      <c r="B29" s="34"/>
+      <c r="C29" s="34"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
     <row r="30" spans="1:6" ht="15">
       <c r="A30" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="C30" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="C30" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
@@ -2755,7 +2755,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="12" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B31" s="12"/>
       <c r="C31" s="12"/>
@@ -2765,7 +2765,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12"/>
@@ -2775,7 +2775,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
@@ -2783,12 +2783,12 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D35" s="2"/>
       <c r="E35" s="2"/>
@@ -2796,7 +2796,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="7" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="2"/>
@@ -2811,24 +2811,24 @@
       <c r="F37" s="2"/>
     </row>
     <row r="38" spans="1:6" s="7" customFormat="1" ht="15">
-      <c r="A38" s="31" t="s">
-        <v>102</v>
-      </c>
-      <c r="B38" s="31"/>
-      <c r="C38" s="31"/>
+      <c r="A38" s="34" t="s">
+        <v>101</v>
+      </c>
+      <c r="B38" s="34"/>
+      <c r="C38" s="34"/>
       <c r="D38" s="2"/>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
     </row>
     <row r="39" spans="1:6" ht="15">
       <c r="A39" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B39" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B39" s="14" t="s">
+      <c r="C39" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2"/>
@@ -2836,12 +2836,12 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D41" s="2"/>
       <c r="E41" s="2"/>
@@ -2849,7 +2849,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
@@ -2857,7 +2857,7 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
@@ -2865,7 +2865,7 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="12" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B44" s="12"/>
       <c r="C44" s="12"/>
@@ -2875,11 +2875,11 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="12" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B45" s="12"/>
       <c r="C45" s="12" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
@@ -2894,24 +2894,24 @@
       <c r="F46" s="2"/>
     </row>
     <row r="47" spans="1:6" ht="15">
-      <c r="A47" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="B47" s="31"/>
-      <c r="C47" s="31"/>
+      <c r="A47" s="34" t="s">
+        <v>109</v>
+      </c>
+      <c r="B47" s="34"/>
+      <c r="C47" s="34"/>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
       <c r="F47" s="2"/>
     </row>
     <row r="48" spans="1:6" ht="15">
       <c r="A48" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B48" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B48" s="14" t="s">
+      <c r="C48" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="C48" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
@@ -2919,7 +2919,7 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B49" s="12"/>
       <c r="C49" s="12"/>
@@ -2929,7 +2929,7 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="12" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B50" s="12"/>
       <c r="C50" s="12"/>
@@ -2939,11 +2939,11 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="12" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B51" s="12"/>
       <c r="C51" s="12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D51" s="2"/>
       <c r="E51" s="2"/>
@@ -2958,24 +2958,24 @@
       <c r="F52" s="2"/>
     </row>
     <row r="53" spans="1:6" ht="15">
-      <c r="A53" s="31" t="s">
-        <v>115</v>
-      </c>
-      <c r="B53" s="31"/>
-      <c r="C53" s="31"/>
+      <c r="A53" s="34" t="s">
+        <v>114</v>
+      </c>
+      <c r="B53" s="34"/>
+      <c r="C53" s="34"/>
       <c r="D53" s="2"/>
       <c r="E53" s="2"/>
       <c r="F53" s="2"/>
     </row>
     <row r="54" spans="1:6" ht="15">
       <c r="A54" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B54" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B54" s="14" t="s">
+      <c r="C54" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="C54" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="D54" s="2"/>
       <c r="E54" s="2"/>
@@ -2983,7 +2983,7 @@
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B55" s="12"/>
       <c r="C55" s="12"/>
@@ -2993,7 +2993,7 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B56" s="12"/>
       <c r="C56" s="12"/>
@@ -3003,7 +3003,7 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="12" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B57" s="12"/>
       <c r="C57" s="12"/>
@@ -3013,7 +3013,7 @@
     </row>
     <row r="58" spans="1:6">
       <c r="A58" s="12" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B58" s="12"/>
       <c r="C58" s="12"/>
@@ -3023,11 +3023,11 @@
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="12" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B59" s="12"/>
       <c r="C59" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="2"/>
@@ -3035,11 +3035,11 @@
     </row>
     <row r="60" spans="1:6">
       <c r="A60" s="12" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B60" s="12"/>
       <c r="C60" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -3054,24 +3054,24 @@
       <c r="F61" s="2"/>
     </row>
     <row r="62" spans="1:6" ht="15">
-      <c r="A62" s="31" t="s">
-        <v>123</v>
-      </c>
-      <c r="B62" s="31"/>
-      <c r="C62" s="31"/>
+      <c r="A62" s="34" t="s">
+        <v>122</v>
+      </c>
+      <c r="B62" s="34"/>
+      <c r="C62" s="34"/>
       <c r="D62" s="2"/>
       <c r="E62" s="2"/>
       <c r="F62" s="2"/>
     </row>
     <row r="63" spans="1:6" ht="15">
       <c r="A63" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="B63" s="14" t="s">
         <v>74</v>
       </c>
-      <c r="B63" s="14" t="s">
+      <c r="C63" s="14" t="s">
         <v>75</v>
-      </c>
-      <c r="C63" s="14" t="s">
-        <v>76</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2"/>
@@ -3079,11 +3079,11 @@
     </row>
     <row r="64" spans="1:6">
       <c r="A64" s="12" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B64" s="12"/>
       <c r="C64" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2"/>
@@ -3091,11 +3091,11 @@
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="12" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B65" s="12"/>
       <c r="C65" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2"/>
@@ -3103,11 +3103,11 @@
     </row>
     <row r="66" spans="1:6">
       <c r="A66" s="12" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B66" s="12"/>
       <c r="C66" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -3115,11 +3115,11 @@
     </row>
     <row r="67" spans="1:6">
       <c r="A67" s="12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B67" s="12"/>
       <c r="C67" s="12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
@@ -3243,61 +3243,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="18">
-      <c r="A1" s="26" t="s">
-        <v>128</v>
-      </c>
-      <c r="B1" s="32"/>
-      <c r="C1" s="32"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="32"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
+      <c r="A1" s="29" t="s">
+        <v>376</v>
+      </c>
+      <c r="B1" s="35"/>
+      <c r="C1" s="35"/>
+      <c r="D1" s="35"/>
+      <c r="E1" s="35"/>
+      <c r="F1" s="35"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="35"/>
+      <c r="I1" s="35"/>
+      <c r="J1" s="35"/>
+      <c r="K1" s="35"/>
     </row>
     <row r="3" spans="1:11" ht="30">
       <c r="A3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>41</v>
-      </c>
       <c r="I3" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="K3" s="3" t="s">
         <v>129</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="4" spans="1:11">
       <c r="A4" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C4" s="2">
         <v>6</v>
@@ -3315,24 +3315,24 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:11">
       <c r="A5" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C5" s="2">
         <v>12</v>
@@ -3350,24 +3350,24 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:11">
       <c r="A6" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C6" s="2">
         <v>5</v>
@@ -3385,24 +3385,24 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:11">
       <c r="A7" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C7" s="2">
         <v>6</v>
@@ -3420,24 +3420,24 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="2" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C8" s="2">
         <v>5</v>
@@ -3455,24 +3455,24 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C9" s="2">
         <v>6</v>
@@ -3490,24 +3490,24 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C10" s="2">
         <v>5</v>
@@ -3525,24 +3525,24 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:11">
       <c r="A11" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C11" s="2">
         <v>6</v>
@@ -3560,24 +3560,24 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12" spans="1:11">
       <c r="A12" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C12" s="2">
         <v>5</v>
@@ -3595,24 +3595,24 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:11">
       <c r="A13" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
@@ -3630,24 +3630,24 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:11">
       <c r="A14" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C14" s="2">
         <v>5</v>
@@ -3665,24 +3665,24 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:11">
       <c r="A15" s="2" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C15" s="2">
         <v>3</v>
@@ -3700,24 +3700,24 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="I15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:11">
       <c r="A16" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C16" s="2">
         <v>1</v>
@@ -3735,24 +3735,24 @@
         <v>7.0000000000000001E-3</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I16" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C17" s="2">
         <v>7.3</v>
@@ -3770,24 +3770,24 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K17" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C18" s="2">
         <v>1</v>
@@ -3805,16 +3805,16 @@
         <v>3.5000000000000001E-3</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -3839,70 +3839,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18">
-      <c r="A1" s="26" t="s">
-        <v>160</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="26"/>
-      <c r="L1" s="26"/>
-      <c r="M1" s="26"/>
-      <c r="N1" s="26"/>
+      <c r="A1" s="29" t="s">
+        <v>158</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
+      <c r="E1" s="29"/>
+      <c r="F1" s="29"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="29"/>
+      <c r="I1" s="29"/>
+      <c r="J1" s="29"/>
+      <c r="K1" s="29"/>
+      <c r="L1" s="29"/>
+      <c r="M1" s="29"/>
+      <c r="N1" s="29"/>
     </row>
     <row r="3" spans="1:14" ht="30">
       <c r="A3" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>161</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>172</v>
-      </c>
       <c r="M3" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="N3" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="28.5">
       <c r="A4" s="2" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B4" s="2"/>
       <c r="C4" s="2"/>
@@ -3916,15 +3916,15 @@
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:14">
       <c r="A5" s="2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
@@ -3939,7 +3939,7 @@
       <c r="L5" s="2"/>
       <c r="M5" s="2"/>
       <c r="N5" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:14">
@@ -3975,65 +3975,65 @@
       <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="15">
-      <c r="A8" s="27" t="s">
-        <v>176</v>
-      </c>
-      <c r="B8" s="27"/>
-      <c r="C8" s="27"/>
-      <c r="D8" s="27"/>
-      <c r="E8" s="27"/>
-      <c r="F8" s="27"/>
-      <c r="G8" s="27"/>
-      <c r="H8" s="27"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="27"/>
-      <c r="L8" s="27"/>
-      <c r="M8" s="27"/>
-      <c r="N8" s="27"/>
+      <c r="A8" s="30" t="s">
+        <v>174</v>
+      </c>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="30"/>
+      <c r="E8" s="30"/>
+      <c r="F8" s="30"/>
+      <c r="G8" s="30"/>
+      <c r="H8" s="30"/>
+      <c r="I8" s="30"/>
+      <c r="J8" s="30"/>
+      <c r="K8" s="30"/>
+      <c r="L8" s="30"/>
+      <c r="M8" s="30"/>
+      <c r="N8" s="30"/>
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="13" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B9" s="13" t="s">
+        <v>175</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="D9" s="13" t="s">
         <v>177</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="E9" s="13" t="s">
         <v>178</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="F9" s="13" t="s">
         <v>179</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="G9" s="13" t="s">
         <v>180</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="H9" s="13" t="s">
         <v>181</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="I9" s="13" t="s">
         <v>182</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="J9" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="K9" s="13" t="s">
         <v>184</v>
       </c>
-      <c r="J9" s="13" t="s">
+      <c r="L9" s="13" t="s">
         <v>185</v>
       </c>
-      <c r="K9" s="13" t="s">
+      <c r="M9" s="13" t="s">
         <v>186</v>
       </c>
-      <c r="L9" s="13" t="s">
+      <c r="N9" s="13" t="s">
         <v>187</v>
-      </c>
-      <c r="M9" s="13" t="s">
-        <v>188</v>
-      </c>
-      <c r="N9" s="13" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="10" spans="1:14">
@@ -7117,151 +7117,151 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="18">
-      <c r="A1" s="26" t="s">
-        <v>190</v>
-      </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
+      <c r="A1" s="29" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="29"/>
+      <c r="C1" s="29"/>
+      <c r="D1" s="29"/>
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>191</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>192</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="28.5">
       <c r="A4" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>311</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>195</v>
-      </c>
-      <c r="B4" s="21" t="s">
-        <v>313</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="15" customFormat="1" ht="71.25">
       <c r="A5" s="2" t="s">
+        <v>356</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>357</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>358</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="D5" s="2" t="s">
         <v>359</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A6" s="2" t="s">
+        <v>360</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>361</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>362</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>365</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>363</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>364</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A7" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>366</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>368</v>
-      </c>
       <c r="C7" s="2" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
     </row>
     <row r="8" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A8" s="2" t="s">
+        <v>368</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>371</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>369</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>370</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>373</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>371</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>372</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="28.5">
       <c r="A9" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>200</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="15" customFormat="1" ht="71.25">
       <c r="A10" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>348</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>350</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>351</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="11" spans="1:4" s="15" customFormat="1" ht="42.75">
       <c r="A11" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>353</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="57">
       <c r="A12" s="2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B12" s="20" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -7269,13 +7269,13 @@
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>204</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -7283,139 +7283,139 @@
         <v>11</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A15" s="19" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="28.5">
       <c r="A16" s="2" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B16" s="23" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:4" s="15" customFormat="1" ht="57">
       <c r="A17" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="B17" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>319</v>
-      </c>
-      <c r="C17" s="2" t="s">
-        <v>320</v>
-      </c>
-      <c r="D17" s="2" t="s">
-        <v>321</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="42.75">
       <c r="A18" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>297</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="D18" s="2" t="s">
         <v>298</v>
-      </c>
-      <c r="C18" s="2" t="s">
-        <v>299</v>
-      </c>
-      <c r="D18" s="2" t="s">
-        <v>300</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="42.75">
       <c r="A19" s="2" t="s">
+        <v>299</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>300</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>301</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="D19" s="2" t="s">
         <v>302</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>303</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>304</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="28.5">
       <c r="A20" s="2" t="s">
+        <v>303</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>304</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>305</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>306</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>307</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>308</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="42.75">
       <c r="A21" s="2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>308</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>311</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="42.75">
       <c r="A22" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="D22" s="2" t="s">
         <v>328</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>329</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="42.75">
       <c r="A23" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="D23" s="2" t="s">
         <v>332</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>333</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -7447,22 +7447,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18">
-      <c r="A1" s="34" t="s">
-        <v>211</v>
-      </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
-      <c r="F1" s="34"/>
-      <c r="G1" s="34"/>
-      <c r="H1" s="34"/>
-      <c r="I1" s="34"/>
-      <c r="J1" s="34"/>
-      <c r="K1" s="34"/>
-      <c r="L1" s="34"/>
-      <c r="M1" s="34"/>
-      <c r="N1" s="34"/>
+      <c r="A1" s="37" t="s">
+        <v>209</v>
+      </c>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
     </row>
     <row r="2" spans="1:14">
       <c r="A2" s="2"/>
@@ -7485,7 +7485,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -7502,10 +7502,10 @@
     </row>
     <row r="4" spans="1:14" ht="57.75">
       <c r="A4" s="10" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B4" s="25" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C4" s="2"/>
       <c r="D4" s="2"/>
@@ -7522,10 +7522,10 @@
     </row>
     <row r="5" spans="1:14" ht="114.75">
       <c r="A5" s="10" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -7542,10 +7542,10 @@
     </row>
     <row r="6" spans="1:14" ht="29.25">
       <c r="A6" s="10" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -7577,79 +7577,79 @@
       <c r="N7" s="2"/>
     </row>
     <row r="8" spans="1:14" ht="15">
-      <c r="A8" s="33" t="s">
-        <v>218</v>
-      </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="33"/>
-      <c r="L8" s="33"/>
-      <c r="M8" s="33"/>
-      <c r="N8" s="33"/>
+      <c r="A8" s="36" t="s">
+        <v>216</v>
+      </c>
+      <c r="B8" s="36"/>
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
+      <c r="J8" s="36"/>
+      <c r="K8" s="36"/>
+      <c r="L8" s="36"/>
+      <c r="M8" s="36"/>
+      <c r="N8" s="36"/>
     </row>
     <row r="9" spans="1:14" ht="30">
       <c r="A9" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C9" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="D9" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="E9" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="F9" s="11" t="s">
         <v>221</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="G9" s="11" t="s">
         <v>222</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="F9" s="11" t="s">
+      <c r="H9" s="11" t="s">
         <v>223</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="I9" s="11" t="s">
         <v>224</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="J9" s="11" t="s">
         <v>225</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="K9" s="11" t="s">
         <v>226</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="L9" s="11" t="s">
         <v>227</v>
       </c>
-      <c r="K9" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>228</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="N9" s="11" t="s">
         <v>229</v>
-      </c>
-      <c r="M9" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="N9" s="11" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="85.5">
       <c r="A10" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>232</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>234</v>
-      </c>
       <c r="D10" s="8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E10" s="8">
         <v>1</v>
@@ -7676,10 +7676,10 @@
         <v>-6.9879518072294089E-2</v>
       </c>
       <c r="M10" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="N10" s="8" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="11" spans="1:14">
@@ -7699,79 +7699,79 @@
       <c r="N11" s="2"/>
     </row>
     <row r="12" spans="1:14" ht="15">
-      <c r="A12" s="33" t="s">
-        <v>237</v>
-      </c>
-      <c r="B12" s="33"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="33"/>
-      <c r="J12" s="33"/>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
-      <c r="N12" s="33"/>
+      <c r="A12" s="36" t="s">
+        <v>235</v>
+      </c>
+      <c r="B12" s="36"/>
+      <c r="C12" s="36"/>
+      <c r="D12" s="36"/>
+      <c r="E12" s="36"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="36"/>
+      <c r="J12" s="36"/>
+      <c r="K12" s="36"/>
+      <c r="L12" s="36"/>
+      <c r="M12" s="36"/>
+      <c r="N12" s="36"/>
     </row>
     <row r="13" spans="1:14" ht="30">
       <c r="A13" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>221</v>
-      </c>
       <c r="D13" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="E13" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="F13" s="11" t="s">
         <v>238</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="G13" s="11" t="s">
         <v>239</v>
       </c>
-      <c r="F13" s="11" t="s">
+      <c r="H13" s="11" t="s">
         <v>240</v>
       </c>
-      <c r="G13" s="11" t="s">
+      <c r="I13" s="11" t="s">
         <v>241</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="J13" s="11" t="s">
         <v>242</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="K13" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="L13" s="11" t="s">
+        <v>229</v>
+      </c>
+      <c r="M13" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="N13" s="11" t="s">
         <v>244</v>
-      </c>
-      <c r="K13" s="11" t="s">
-        <v>230</v>
-      </c>
-      <c r="L13" s="11" t="s">
-        <v>231</v>
-      </c>
-      <c r="M13" s="11" t="s">
-        <v>245</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="14" spans="1:14" ht="28.5">
       <c r="A14" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>247</v>
       </c>
-      <c r="B14" s="8" t="s">
+      <c r="D14" s="8" t="s">
         <v>248</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="D14" s="8" t="s">
-        <v>250</v>
       </c>
       <c r="E14" s="8">
         <v>490.11</v>
@@ -7792,30 +7792,30 @@
         <v>-8.4128576014130138E-2</v>
       </c>
       <c r="K14" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L14" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M14" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N14" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M14" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N14" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="28.5">
       <c r="A15" s="8" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E15" s="8">
         <v>490.11</v>
@@ -7836,30 +7836,30 @@
         <v>-0.1649644901525206</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L15" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N15" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M15" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N15" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="16" spans="1:14" ht="28.5">
       <c r="A16" s="8" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B16" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>248</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>257</v>
-      </c>
-      <c r="D16" s="8" t="s">
-        <v>250</v>
       </c>
       <c r="E16" s="8">
         <v>428.4</v>
@@ -7880,30 +7880,30 @@
         <v>1.6132982587243029E-2</v>
       </c>
       <c r="K16" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L16" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M16" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N16" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M16" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N16" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="28.5">
       <c r="A17" s="8" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B17" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="D17" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E17" s="8">
         <v>428.4</v>
@@ -7924,30 +7924,30 @@
         <v>8.7237397338995933E-3</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L17" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M17" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N17" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M17" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N17" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="28.5">
       <c r="A18" s="8" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B18" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>258</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>248</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>260</v>
-      </c>
-      <c r="D18" s="8" t="s">
-        <v>250</v>
       </c>
       <c r="E18" s="8">
         <v>484.63</v>
@@ -7968,30 +7968,30 @@
         <v>-4.5187050999701966E-3</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L18" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M18" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N18" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M18" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N18" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="28.5">
       <c r="A19" s="8" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="D19" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E19" s="8">
         <v>484.63</v>
@@ -8012,30 +8012,30 @@
         <v>-4.0114456608485519E-3</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L19" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N19" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M19" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N19" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="28.5">
       <c r="A20" s="8" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B20" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>248</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>263</v>
-      </c>
-      <c r="D20" s="8" t="s">
-        <v>250</v>
       </c>
       <c r="E20" s="8">
         <v>413.02</v>
@@ -8056,30 +8056,30 @@
         <v>-6.0227292075755966E-3</v>
       </c>
       <c r="K20" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L20" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M20" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N20" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M20" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N20" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="28.5">
       <c r="A21" s="8" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="D21" s="8" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="E21" s="8">
         <v>413.02</v>
@@ -8100,16 +8100,16 @@
         <v>4.72329903258944E-4</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="L21" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M21" s="8" t="s">
+        <v>250</v>
+      </c>
+      <c r="N21" s="8" t="s">
         <v>251</v>
-      </c>
-      <c r="M21" s="8" t="s">
-        <v>252</v>
-      </c>
-      <c r="N21" s="8" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="22" spans="1:14">
@@ -8145,29 +8145,29 @@
       <c r="N23" s="2"/>
     </row>
     <row r="24" spans="1:14" ht="15">
-      <c r="A24" s="33" t="s">
-        <v>265</v>
-      </c>
-      <c r="B24" s="33"/>
-      <c r="C24" s="33"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="33"/>
+      <c r="A24" s="36" t="s">
+        <v>263</v>
+      </c>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
     </row>
     <row r="25" spans="1:14" ht="30">
       <c r="A25" s="11" t="s">
+        <v>264</v>
+      </c>
+      <c r="B25" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>265</v>
+      </c>
+      <c r="D25" s="11" t="s">
         <v>266</v>
       </c>
-      <c r="B25" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="C25" s="11" t="s">
+      <c r="E25" s="11" t="s">
         <v>267</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>268</v>
-      </c>
-      <c r="E25" s="11" t="s">
-        <v>269</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -8181,19 +8181,19 @@
     </row>
     <row r="26" spans="1:14" ht="85.5">
       <c r="A26" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="B26" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C26" s="9" t="s">
         <v>270</v>
       </c>
-      <c r="B26" s="9" t="s">
+      <c r="D26" s="9" t="s">
         <v>271</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="E26" s="9" t="s">
         <v>272</v>
-      </c>
-      <c r="D26" s="9" t="s">
-        <v>273</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>274</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -8207,19 +8207,19 @@
     </row>
     <row r="27" spans="1:14" ht="85.5">
       <c r="A27" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="C27" s="9" t="s">
         <v>275</v>
       </c>
-      <c r="B27" s="9" t="s">
+      <c r="D27" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="E27" s="9" t="s">
         <v>277</v>
-      </c>
-      <c r="D27" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>279</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -8233,19 +8233,19 @@
     </row>
     <row r="28" spans="1:14" ht="71.25">
       <c r="A28" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="B28" s="9" t="s">
+        <v>279</v>
+      </c>
+      <c r="C28" s="9" t="s">
         <v>280</v>
       </c>
-      <c r="B28" s="9" t="s">
+      <c r="D28" s="9" t="s">
         <v>281</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="E28" s="9" t="s">
         <v>282</v>
-      </c>
-      <c r="D28" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>284</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
@@ -8290,17 +8290,17 @@
       <c r="N30" s="2"/>
     </row>
     <row r="31" spans="1:14" ht="15">
-      <c r="A31" s="33" t="s">
-        <v>285</v>
-      </c>
-      <c r="B31" s="33"/>
+      <c r="A31" s="36" t="s">
+        <v>283</v>
+      </c>
+      <c r="B31" s="36"/>
     </row>
     <row r="32" spans="1:14" ht="15">
       <c r="A32" s="11" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -8317,10 +8317,10 @@
     </row>
     <row r="33" spans="1:14" ht="57">
       <c r="A33" s="2" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B33" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -8337,10 +8337,10 @@
     </row>
     <row r="34" spans="1:14" ht="57">
       <c r="A34" s="2" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="B34" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -8357,10 +8357,10 @@
     </row>
     <row r="35" spans="1:14" ht="42.75">
       <c r="A35" s="2" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B35" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -8377,10 +8377,10 @@
     </row>
     <row r="36" spans="1:14" ht="57">
       <c r="A36" s="2" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="B36" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -8397,10 +8397,10 @@
     </row>
     <row r="37" spans="1:14" ht="57">
       <c r="A37" s="2" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B37" s="8" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>

</xml_diff>